<commit_message>
End of session — Timeline updated to April 1, 2026
Extended Iran War Timeline through 1 April 2026 with two major updates:
- Trump announces US campaign wind-down in 2–3 weeks regardless of deal; message to European allies on Hormuz; national address scheduled for April 2
- Iranian President Pezeshkian's March 31 statement: Iran has 'necessary will' to end war provided security guarantees received

Research verified via multiple sources (Al Jazeera, BBC, CNN) with all links in HTML anchor format.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hseea/HSE Actions List.xlsx
+++ b/hseea/HSE Actions List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SteveIrwin\terminai\hseea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16B5A6C9-026B-4366-A733-228627A3FFC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3644DAB7-8C12-4974-B0CC-C187B5DF7242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A67E721E-67E3-4729-8C79-A57CFF14FB61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A67E721E-67E3-4729-8C79-A57CFF14FB61}"/>
   </bookViews>
   <sheets>
     <sheet name="HSE Actions List" sheetId="1" r:id="rId1"/>
@@ -1470,14 +1470,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1487,9 +1486,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
@@ -1537,11 +1536,9 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="55" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="61" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="62" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="63" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1"/>
@@ -3559,7 +3556,7 @@
         <v>2</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>16</v>
+        <v>87</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -4683,552 +4680,525 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
-      <c r="AA3" s="4"/>
-      <c r="AB3" s="5"/>
+      <c r="AB3" s="4"/>
     </row>
     <row r="4" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="6"/>
-      <c r="Z4" s="6"/>
-      <c r="AA4" s="6"/>
-      <c r="AB4" s="7"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="5"/>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="5"/>
+      <c r="AA4" s="5"/>
+      <c r="AB4" s="6"/>
     </row>
     <row r="5" spans="1:96" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="9"/>
-      <c r="F5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="D6" s="9"/>
-      <c r="E6" s="8"/>
-      <c r="G6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="7"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="C7" s="9"/>
-      <c r="D7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="C8" s="10"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="11"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
-      <c r="S9" s="13"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="13"/>
-      <c r="W9" s="13"/>
-      <c r="X9" s="13"/>
-      <c r="Y9" s="13"/>
-      <c r="Z9" s="13"/>
-      <c r="AA9" s="13"/>
-      <c r="AB9" s="13"/>
-      <c r="AC9" s="13"/>
-      <c r="AD9" s="13"/>
-      <c r="AE9" s="13"/>
-      <c r="AF9" s="13"/>
-      <c r="AG9" s="13"/>
-      <c r="AH9" s="13"/>
-      <c r="AI9" s="13"/>
-      <c r="AJ9" s="13"/>
-      <c r="AK9" s="13"/>
-      <c r="AL9" s="13"/>
-      <c r="AM9" s="13"/>
-      <c r="AN9" s="13"/>
-      <c r="AO9" s="13"/>
-      <c r="AP9" s="13"/>
-      <c r="AQ9" s="13"/>
-      <c r="AR9" s="13"/>
-      <c r="AS9" s="13"/>
-      <c r="AT9" s="13"/>
-      <c r="AU9" s="13"/>
-      <c r="AV9" s="13"/>
-      <c r="AW9" s="13"/>
-      <c r="AX9" s="13"/>
-      <c r="AY9" s="13"/>
-      <c r="AZ9" s="13"/>
-      <c r="BA9" s="13"/>
-      <c r="BB9" s="13"/>
-      <c r="BC9" s="13"/>
-      <c r="BD9" s="13"/>
-      <c r="BE9" s="13"/>
-      <c r="BF9" s="13"/>
-      <c r="BG9" s="13"/>
-      <c r="BH9" s="13"/>
-      <c r="BI9" s="13"/>
-      <c r="BJ9" s="13"/>
-      <c r="BK9" s="13"/>
-      <c r="BL9" s="13"/>
-      <c r="BM9" s="13"/>
-      <c r="BN9" s="13"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="12"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
+      <c r="Y9" s="12"/>
+      <c r="Z9" s="12"/>
+      <c r="AA9" s="12"/>
+      <c r="AB9" s="12"/>
+      <c r="AC9" s="12"/>
+      <c r="AD9" s="12"/>
+      <c r="AE9" s="12"/>
+      <c r="AF9" s="12"/>
+      <c r="AG9" s="12"/>
+      <c r="AH9" s="12"/>
+      <c r="AI9" s="12"/>
+      <c r="AJ9" s="12"/>
+      <c r="AK9" s="12"/>
+      <c r="AL9" s="12"/>
+      <c r="AM9" s="12"/>
+      <c r="AN9" s="12"/>
+      <c r="AO9" s="12"/>
+      <c r="AP9" s="12"/>
+      <c r="AQ9" s="12"/>
+      <c r="AR9" s="12"/>
+      <c r="AS9" s="12"/>
+      <c r="AT9" s="12"/>
+      <c r="AU9" s="12"/>
+      <c r="AV9" s="12"/>
+      <c r="AW9" s="12"/>
+      <c r="AX9" s="12"/>
+      <c r="AY9" s="12"/>
+      <c r="AZ9" s="12"/>
+      <c r="BA9" s="12"/>
+      <c r="BB9" s="12"/>
+      <c r="BC9" s="12"/>
+      <c r="BD9" s="12"/>
+      <c r="BE9" s="12"/>
+      <c r="BF9" s="12"/>
+      <c r="BG9" s="12"/>
+      <c r="BH9" s="12"/>
+      <c r="BI9" s="12"/>
+      <c r="BJ9" s="12"/>
+      <c r="BK9" s="12"/>
+      <c r="BL9" s="12"/>
+      <c r="BM9" s="12"/>
+      <c r="BN9" s="12"/>
     </row>
     <row r="10" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="14"/>
-      <c r="S10" s="14"/>
-      <c r="T10" s="14"/>
-      <c r="U10" s="14"/>
-      <c r="V10" s="14"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="14"/>
-      <c r="Y10" s="14"/>
-      <c r="Z10" s="14"/>
-      <c r="AA10" s="14"/>
-      <c r="AB10" s="14"/>
-      <c r="AC10" s="14"/>
-      <c r="AD10" s="14"/>
-      <c r="AE10" s="14"/>
-      <c r="AF10" s="14"/>
-      <c r="AG10" s="14"/>
-      <c r="AH10" s="14"/>
-      <c r="AI10" s="14"/>
-      <c r="AJ10" s="14"/>
-      <c r="AK10" s="14"/>
-      <c r="AL10" s="14"/>
-      <c r="AM10" s="14"/>
-      <c r="AN10" s="14"/>
-      <c r="AO10" s="14"/>
-      <c r="AP10" s="14"/>
-      <c r="AQ10" s="14"/>
-      <c r="AR10" s="14"/>
-      <c r="AS10" s="14"/>
-      <c r="AT10" s="14"/>
-      <c r="AU10" s="14"/>
-      <c r="AV10" s="14"/>
-      <c r="AW10" s="14"/>
-      <c r="AX10" s="14"/>
-      <c r="AY10" s="14"/>
-      <c r="AZ10" s="14"/>
-      <c r="BA10" s="14"/>
-      <c r="BB10" s="14"/>
-      <c r="BC10" s="14"/>
-      <c r="BD10" s="14"/>
-      <c r="BE10" s="14"/>
-      <c r="BF10" s="14"/>
-      <c r="BG10" s="14"/>
-      <c r="BH10" s="14"/>
-      <c r="BI10" s="14"/>
-      <c r="BJ10" s="14"/>
-      <c r="BK10" s="14"/>
-      <c r="BL10" s="14"/>
-      <c r="BM10" s="14"/>
-      <c r="BN10" s="14"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="13"/>
+      <c r="AI10" s="13"/>
+      <c r="AJ10" s="13"/>
+      <c r="AK10" s="13"/>
+      <c r="AL10" s="13"/>
+      <c r="AM10" s="13"/>
+      <c r="AN10" s="13"/>
+      <c r="AO10" s="13"/>
+      <c r="AP10" s="13"/>
+      <c r="AQ10" s="13"/>
+      <c r="AR10" s="13"/>
+      <c r="AS10" s="13"/>
+      <c r="AT10" s="13"/>
+      <c r="AU10" s="13"/>
+      <c r="AV10" s="13"/>
+      <c r="AW10" s="13"/>
+      <c r="AX10" s="13"/>
+      <c r="AY10" s="13"/>
+      <c r="AZ10" s="13"/>
+      <c r="BA10" s="13"/>
+      <c r="BB10" s="13"/>
+      <c r="BC10" s="13"/>
+      <c r="BD10" s="13"/>
+      <c r="BE10" s="13"/>
+      <c r="BF10" s="13"/>
+      <c r="BG10" s="13"/>
+      <c r="BH10" s="13"/>
+      <c r="BI10" s="13"/>
+      <c r="BJ10" s="13"/>
+      <c r="BK10" s="13"/>
+      <c r="BL10" s="13"/>
+      <c r="BM10" s="13"/>
+      <c r="BN10" s="13"/>
     </row>
     <row r="11" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="72"/>
-      <c r="Q11" s="72"/>
-      <c r="R11" s="72"/>
-      <c r="S11" s="72"/>
-      <c r="T11" s="72"/>
-      <c r="U11" s="72"/>
-      <c r="V11" s="72"/>
-      <c r="W11" s="72"/>
-      <c r="X11" s="72"/>
-      <c r="Y11" s="72"/>
-      <c r="Z11" s="72"/>
-      <c r="AA11" s="72"/>
-      <c r="AB11" s="72"/>
-      <c r="AC11" s="72"/>
-      <c r="AD11" s="72"/>
-      <c r="AE11" s="72"/>
-      <c r="AF11" s="72"/>
-      <c r="AG11" s="72"/>
-      <c r="AH11" s="72"/>
-      <c r="AI11" s="72"/>
-      <c r="AJ11" s="72"/>
-      <c r="AK11" s="72"/>
-      <c r="AL11" s="72"/>
-      <c r="AM11" s="72"/>
-      <c r="AN11" s="72"/>
-      <c r="AO11" s="72"/>
-      <c r="AP11" s="72"/>
-      <c r="AQ11" s="72"/>
-      <c r="AR11" s="72"/>
-      <c r="AS11" s="72"/>
-      <c r="AT11" s="72"/>
-      <c r="AU11" s="72"/>
-      <c r="AV11" s="14"/>
-      <c r="AW11" s="14"/>
-      <c r="AX11" s="14"/>
-      <c r="AY11" s="14"/>
-      <c r="AZ11" s="14"/>
-      <c r="BA11" s="14"/>
-      <c r="BB11" s="14"/>
-      <c r="BC11" s="14"/>
-      <c r="BD11" s="14"/>
-      <c r="BE11" s="14"/>
-      <c r="BF11" s="14"/>
-      <c r="BG11" s="14"/>
-      <c r="BH11" s="14"/>
-      <c r="BI11" s="14"/>
-      <c r="BJ11" s="14"/>
-      <c r="BK11" s="14"/>
-      <c r="BL11" s="14"/>
-      <c r="BM11" s="14"/>
-      <c r="BN11" s="14"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="69"/>
+      <c r="Q11" s="69"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="69"/>
+      <c r="T11" s="69"/>
+      <c r="U11" s="69"/>
+      <c r="V11" s="69"/>
+      <c r="W11" s="69"/>
+      <c r="X11" s="69"/>
+      <c r="Y11" s="69"/>
+      <c r="Z11" s="69"/>
+      <c r="AA11" s="69"/>
+      <c r="AB11" s="69"/>
+      <c r="AC11" s="69"/>
+      <c r="AD11" s="69"/>
+      <c r="AE11" s="69"/>
+      <c r="AF11" s="69"/>
+      <c r="AG11" s="69"/>
+      <c r="AH11" s="69"/>
+      <c r="AI11" s="69"/>
+      <c r="AJ11" s="69"/>
+      <c r="AK11" s="69"/>
+      <c r="AL11" s="69"/>
+      <c r="AM11" s="69"/>
+      <c r="AN11" s="69"/>
+      <c r="AO11" s="69"/>
+      <c r="AP11" s="69"/>
+      <c r="AQ11" s="69"/>
+      <c r="AR11" s="69"/>
+      <c r="AS11" s="69"/>
+      <c r="AT11" s="69"/>
+      <c r="AU11" s="69"/>
+      <c r="AV11" s="13"/>
+      <c r="AW11" s="13"/>
+      <c r="AX11" s="13"/>
+      <c r="AY11" s="13"/>
+      <c r="AZ11" s="13"/>
+      <c r="BA11" s="13"/>
+      <c r="BB11" s="13"/>
+      <c r="BC11" s="13"/>
+      <c r="BD11" s="13"/>
+      <c r="BE11" s="13"/>
+      <c r="BF11" s="13"/>
+      <c r="BG11" s="13"/>
+      <c r="BH11" s="13"/>
+      <c r="BI11" s="13"/>
+      <c r="BJ11" s="13"/>
+      <c r="BK11" s="13"/>
+      <c r="BL11" s="13"/>
+      <c r="BM11" s="13"/>
+      <c r="BN11" s="13"/>
     </row>
     <row r="12" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="61"/>
-      <c r="Q12" s="61"/>
-      <c r="R12" s="61"/>
-      <c r="S12" s="61"/>
-      <c r="T12" s="61"/>
-      <c r="U12" s="61"/>
-      <c r="V12" s="61"/>
-      <c r="W12" s="61"/>
-      <c r="X12" s="61"/>
-      <c r="Y12" s="61"/>
-      <c r="Z12" s="61"/>
-      <c r="AA12" s="61"/>
-      <c r="AB12" s="61"/>
-      <c r="AC12" s="61"/>
-      <c r="AD12" s="61"/>
-      <c r="AE12" s="61"/>
-      <c r="AF12" s="61"/>
-      <c r="AG12" s="61"/>
-      <c r="AH12" s="61"/>
-      <c r="AI12" s="61"/>
-      <c r="AJ12" s="61"/>
-      <c r="AK12" s="61"/>
-      <c r="AL12" s="61"/>
-      <c r="AM12" s="61"/>
-      <c r="AN12" s="61"/>
-      <c r="AO12" s="61"/>
-      <c r="AP12" s="61"/>
-      <c r="AQ12" s="61"/>
-      <c r="AR12" s="61"/>
-      <c r="AS12" s="61"/>
-      <c r="AT12" s="61"/>
-      <c r="AU12" s="61"/>
-      <c r="AV12" s="61"/>
-      <c r="AW12" s="61"/>
-      <c r="AX12" s="61"/>
-      <c r="AY12" s="61"/>
-      <c r="AZ12" s="61"/>
-      <c r="BA12" s="61"/>
-      <c r="BB12" s="61"/>
-      <c r="BC12" s="61"/>
-      <c r="BD12" s="61"/>
-      <c r="BE12" s="61"/>
-      <c r="BF12" s="62"/>
-      <c r="BG12" s="14"/>
-      <c r="BH12" s="14"/>
-      <c r="BI12" s="14"/>
-      <c r="BJ12" s="14"/>
-      <c r="BK12" s="14"/>
-      <c r="BL12" s="14"/>
-      <c r="BM12" s="14"/>
-      <c r="BN12" s="14"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="60"/>
+      <c r="Q12" s="60"/>
+      <c r="R12" s="60"/>
+      <c r="S12" s="60"/>
+      <c r="T12" s="60"/>
+      <c r="U12" s="60"/>
+      <c r="V12" s="60"/>
+      <c r="W12" s="60"/>
+      <c r="X12" s="60"/>
+      <c r="Y12" s="60"/>
+      <c r="Z12" s="60"/>
+      <c r="AA12" s="60"/>
+      <c r="AB12" s="60"/>
+      <c r="AC12" s="60"/>
+      <c r="AD12" s="60"/>
+      <c r="AE12" s="60"/>
+      <c r="AF12" s="60"/>
+      <c r="AG12" s="60"/>
+      <c r="AH12" s="60"/>
+      <c r="AI12" s="60"/>
+      <c r="AJ12" s="60"/>
+      <c r="AK12" s="60"/>
+      <c r="AL12" s="60"/>
+      <c r="AM12" s="60"/>
+      <c r="AN12" s="60"/>
+      <c r="AO12" s="60"/>
+      <c r="AP12" s="60"/>
+      <c r="AQ12" s="60"/>
+      <c r="AR12" s="60"/>
+      <c r="AS12" s="60"/>
+      <c r="AT12" s="60"/>
+      <c r="AU12" s="60"/>
+      <c r="AV12" s="60"/>
+      <c r="AW12" s="60"/>
+      <c r="AX12" s="60"/>
+      <c r="AY12" s="60"/>
+      <c r="AZ12" s="60"/>
+      <c r="BA12" s="60"/>
+      <c r="BB12" s="60"/>
+      <c r="BC12" s="60"/>
+      <c r="BD12" s="60"/>
+      <c r="BE12" s="60"/>
+      <c r="BF12" s="61"/>
+      <c r="BG12" s="13"/>
+      <c r="BH12" s="13"/>
+      <c r="BI12" s="13"/>
+      <c r="BJ12" s="13"/>
+      <c r="BK12" s="13"/>
+      <c r="BL12" s="13"/>
+      <c r="BM12" s="13"/>
+      <c r="BN12" s="13"/>
     </row>
     <row r="13" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
-      <c r="S13" s="15"/>
-      <c r="T13" s="15"/>
-      <c r="U13" s="15"/>
-      <c r="V13" s="15"/>
-      <c r="W13" s="15"/>
-      <c r="X13" s="15"/>
-      <c r="Y13" s="15"/>
-      <c r="Z13" s="15"/>
-      <c r="AA13" s="15"/>
-      <c r="AB13" s="15"/>
-      <c r="AC13" s="15"/>
-      <c r="AD13" s="15"/>
-      <c r="AE13" s="15"/>
-      <c r="AF13" s="15"/>
-      <c r="AG13" s="15"/>
-      <c r="AH13" s="15"/>
-      <c r="AI13" s="15"/>
-      <c r="AJ13" s="15"/>
-      <c r="AK13" s="15"/>
-      <c r="AL13" s="15"/>
-      <c r="AM13" s="15"/>
-      <c r="AN13" s="15"/>
-      <c r="AO13" s="15"/>
-      <c r="AP13" s="15"/>
-      <c r="AQ13" s="15"/>
-      <c r="AR13" s="15"/>
-      <c r="AS13" s="15"/>
-      <c r="AT13" s="15"/>
-      <c r="AU13" s="15"/>
-      <c r="AV13" s="15"/>
-      <c r="AW13" s="15"/>
-      <c r="AX13" s="15"/>
-      <c r="AY13" s="15"/>
-      <c r="AZ13" s="15"/>
-      <c r="BA13" s="15"/>
-      <c r="BB13" s="15"/>
-      <c r="BC13" s="15"/>
-      <c r="BD13" s="15"/>
-      <c r="BE13" s="15"/>
-      <c r="BF13" s="63"/>
-      <c r="BG13" s="15"/>
-      <c r="BH13" s="15"/>
-      <c r="BI13" s="15"/>
-      <c r="BJ13" s="15"/>
-      <c r="BK13" s="15"/>
-      <c r="BL13" s="15"/>
-      <c r="BM13" s="15"/>
-      <c r="BN13" s="15"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="14"/>
+      <c r="S13" s="14"/>
+      <c r="T13" s="14"/>
+      <c r="U13" s="14"/>
+      <c r="V13" s="14"/>
+      <c r="W13" s="14"/>
+      <c r="X13" s="14"/>
+      <c r="Y13" s="14"/>
+      <c r="Z13" s="14"/>
+      <c r="AA13" s="14"/>
+      <c r="AB13" s="14"/>
+      <c r="AC13" s="14"/>
+      <c r="AD13" s="14"/>
+      <c r="AE13" s="14"/>
+      <c r="AF13" s="14"/>
+      <c r="AG13" s="14"/>
+      <c r="AH13" s="14"/>
+      <c r="AI13" s="14"/>
+      <c r="AJ13" s="14"/>
+      <c r="AK13" s="14"/>
+      <c r="AL13" s="14"/>
+      <c r="AM13" s="14"/>
+      <c r="AN13" s="14"/>
+      <c r="AO13" s="14"/>
+      <c r="AP13" s="14"/>
+      <c r="AQ13" s="14"/>
+      <c r="AR13" s="14"/>
+      <c r="AS13" s="14"/>
+      <c r="AT13" s="14"/>
+      <c r="AU13" s="14"/>
+      <c r="AV13" s="14"/>
+      <c r="AW13" s="14"/>
+      <c r="AX13" s="14"/>
+      <c r="AY13" s="14"/>
+      <c r="AZ13" s="14"/>
+      <c r="BA13" s="14"/>
+      <c r="BB13" s="14"/>
+      <c r="BC13" s="14"/>
+      <c r="BD13" s="14"/>
+      <c r="BE13" s="14"/>
+      <c r="BF13" s="62"/>
+      <c r="BG13" s="14"/>
+      <c r="BH13" s="14"/>
+      <c r="BI13" s="14"/>
+      <c r="BJ13" s="14"/>
+      <c r="BK13" s="14"/>
+      <c r="BL13" s="14"/>
+      <c r="BM13" s="14"/>
+      <c r="BN13" s="14"/>
     </row>
     <row r="14" spans="1:96" ht="7.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
-      <c r="O14" s="17"/>
-      <c r="P14" s="17"/>
-      <c r="Q14" s="17"/>
-      <c r="R14" s="17"/>
-      <c r="S14" s="17"/>
-      <c r="T14" s="17"/>
-      <c r="U14" s="17"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="17"/>
-      <c r="X14" s="17"/>
-      <c r="Y14" s="17"/>
-      <c r="Z14" s="17"/>
-      <c r="AA14" s="17"/>
-      <c r="AB14" s="17"/>
-      <c r="AC14" s="17"/>
-      <c r="AD14" s="17"/>
-      <c r="AE14" s="17"/>
-      <c r="AF14" s="17"/>
-      <c r="AG14" s="17"/>
-      <c r="AH14" s="17"/>
-      <c r="AI14" s="17"/>
-      <c r="AJ14" s="17"/>
-      <c r="AK14" s="17"/>
-      <c r="AL14" s="17"/>
-      <c r="AM14" s="17"/>
-      <c r="AN14" s="17"/>
-      <c r="AO14" s="17"/>
-      <c r="AP14" s="17"/>
-      <c r="AQ14" s="17"/>
-      <c r="AR14" s="17"/>
-      <c r="AS14" s="17"/>
-      <c r="AT14" s="17"/>
-      <c r="AU14" s="64"/>
-      <c r="AV14" s="64"/>
-      <c r="AW14" s="64"/>
-      <c r="AX14" s="64"/>
-      <c r="AY14" s="64"/>
-      <c r="AZ14" s="64"/>
-      <c r="BA14" s="64"/>
-      <c r="BB14" s="64"/>
-      <c r="BC14" s="64"/>
-      <c r="BD14" s="64"/>
-      <c r="BE14" s="64"/>
-      <c r="BF14" s="65"/>
-      <c r="BG14" s="17"/>
-      <c r="BH14" s="17"/>
-      <c r="BI14" s="17"/>
-      <c r="BJ14" s="17"/>
-      <c r="BK14" s="17"/>
-      <c r="BL14" s="17"/>
-      <c r="BM14" s="17"/>
-      <c r="BN14" s="17"/>
-    </row>
-    <row r="15" spans="1:96" s="16" customFormat="1" ht="10.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="16"/>
+      <c r="U14" s="16"/>
+      <c r="V14" s="16"/>
+      <c r="W14" s="16"/>
+      <c r="X14" s="16"/>
+      <c r="Y14" s="16"/>
+      <c r="Z14" s="16"/>
+      <c r="AA14" s="16"/>
+      <c r="AB14" s="16"/>
+      <c r="AC14" s="16"/>
+      <c r="AD14" s="16"/>
+      <c r="AE14" s="16"/>
+      <c r="AF14" s="16"/>
+      <c r="AG14" s="16"/>
+      <c r="AH14" s="16"/>
+      <c r="AI14" s="16"/>
+      <c r="AJ14" s="16"/>
+      <c r="AK14" s="16"/>
+      <c r="AL14" s="16"/>
+      <c r="AM14" s="16"/>
+      <c r="AN14" s="16"/>
+      <c r="AO14" s="16"/>
+      <c r="AP14" s="16"/>
+      <c r="AQ14" s="16"/>
+      <c r="AR14" s="16"/>
+      <c r="AS14" s="16"/>
+      <c r="AT14" s="16"/>
+      <c r="AU14" s="16"/>
+      <c r="AV14" s="16"/>
+      <c r="AW14" s="16"/>
+      <c r="AX14" s="16"/>
+      <c r="AY14" s="16"/>
+      <c r="AZ14" s="16"/>
+      <c r="BA14" s="16"/>
+      <c r="BB14" s="16"/>
+      <c r="BC14" s="16"/>
+      <c r="BD14" s="16"/>
+      <c r="BE14" s="16"/>
+      <c r="BF14" s="63"/>
+      <c r="BG14" s="16"/>
+      <c r="BH14" s="16"/>
+      <c r="BI14" s="16"/>
+      <c r="BJ14" s="16"/>
+      <c r="BK14" s="16"/>
+      <c r="BL14" s="16"/>
+      <c r="BM14" s="16"/>
+      <c r="BN14" s="16"/>
+    </row>
+    <row r="15" spans="1:96" s="15" customFormat="1" ht="10.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="18"/>
-      <c r="P15" s="18"/>
-      <c r="Q15" s="18"/>
-      <c r="R15" s="18"/>
-      <c r="S15" s="18"/>
-      <c r="T15" s="18"/>
-      <c r="U15" s="18"/>
-      <c r="V15" s="18"/>
-      <c r="W15" s="18"/>
-      <c r="X15" s="18"/>
-      <c r="Y15" s="18"/>
-      <c r="Z15" s="18"/>
-      <c r="AA15" s="18"/>
-      <c r="AB15" s="18"/>
-      <c r="AC15" s="18"/>
-      <c r="AD15" s="18"/>
-      <c r="AE15" s="18"/>
-      <c r="AF15" s="18"/>
-      <c r="AG15" s="18"/>
-      <c r="AH15" s="18"/>
-      <c r="AI15" s="18"/>
-      <c r="AJ15" s="18"/>
-      <c r="AK15" s="18"/>
-      <c r="AL15" s="18"/>
-      <c r="AM15" s="18"/>
-      <c r="AN15" s="18"/>
-      <c r="AO15" s="18"/>
-      <c r="AP15" s="18"/>
-      <c r="AQ15" s="18"/>
-      <c r="AR15" s="18"/>
-      <c r="AS15" s="18"/>
-      <c r="AT15" s="18"/>
-      <c r="AU15" s="18"/>
-      <c r="AV15" s="18"/>
-      <c r="AW15" s="18"/>
-      <c r="AX15" s="18"/>
-      <c r="AY15" s="18"/>
-      <c r="AZ15" s="18"/>
-      <c r="BA15" s="18"/>
-      <c r="BB15" s="18"/>
-      <c r="BC15" s="18"/>
-      <c r="BD15" s="18"/>
-      <c r="BE15" s="18"/>
-      <c r="BF15" s="66"/>
-      <c r="BG15" s="18"/>
-      <c r="BH15" s="18"/>
-      <c r="BI15" s="18"/>
-      <c r="BJ15" s="18"/>
-      <c r="BK15" s="18"/>
-      <c r="BL15" s="18"/>
-      <c r="BM15" s="18"/>
-      <c r="BN15" s="18"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17"/>
+      <c r="T15" s="17"/>
+      <c r="U15" s="17"/>
+      <c r="V15" s="17"/>
+      <c r="W15" s="17"/>
+      <c r="X15" s="17"/>
+      <c r="Y15" s="17"/>
+      <c r="Z15" s="17"/>
+      <c r="AA15" s="17"/>
+      <c r="AB15" s="17"/>
+      <c r="AC15" s="17"/>
+      <c r="AD15" s="17"/>
+      <c r="AE15" s="17"/>
+      <c r="AF15" s="17"/>
+      <c r="AG15" s="17"/>
+      <c r="AH15" s="17"/>
+      <c r="AI15" s="17"/>
+      <c r="AJ15" s="17"/>
+      <c r="AK15" s="17"/>
+      <c r="AL15" s="17"/>
+      <c r="AM15" s="17"/>
+      <c r="AN15" s="17"/>
+      <c r="AO15" s="17"/>
+      <c r="AP15" s="17"/>
+      <c r="AQ15" s="17"/>
+      <c r="AR15" s="17"/>
+      <c r="AS15" s="17"/>
+      <c r="AT15" s="17"/>
+      <c r="AU15" s="17"/>
+      <c r="AV15" s="17"/>
+      <c r="AW15" s="17"/>
+      <c r="AX15" s="17"/>
+      <c r="AY15" s="17"/>
+      <c r="AZ15" s="17"/>
+      <c r="BA15" s="17"/>
+      <c r="BB15" s="17"/>
+      <c r="BC15" s="17"/>
+      <c r="BD15" s="17"/>
+      <c r="BE15" s="17"/>
+      <c r="BF15" s="64"/>
+      <c r="BG15" s="17"/>
+      <c r="BH15" s="17"/>
+      <c r="BI15" s="17"/>
+      <c r="BJ15" s="17"/>
+      <c r="BK15" s="17"/>
+      <c r="BL15" s="17"/>
+      <c r="BM15" s="17"/>
+      <c r="BN15" s="17"/>
       <c r="BO15"/>
       <c r="BP15"/>
       <c r="BQ15"/>
@@ -5261,608 +5231,608 @@
       <c r="CR15"/>
     </row>
     <row r="16" spans="1:96" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
-      <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="17"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="17"/>
-      <c r="U16" s="17"/>
-      <c r="V16" s="17"/>
-      <c r="W16" s="17"/>
-      <c r="X16" s="17"/>
-      <c r="Y16" s="17"/>
-      <c r="Z16" s="17"/>
-      <c r="AA16" s="17"/>
-      <c r="AB16" s="17"/>
-      <c r="AC16" s="17"/>
-      <c r="AD16" s="17"/>
-      <c r="AE16" s="17"/>
-      <c r="AF16" s="17"/>
-      <c r="AG16" s="17"/>
-      <c r="AH16" s="17"/>
-      <c r="AI16" s="17"/>
-      <c r="AJ16" s="17"/>
-      <c r="AK16" s="17"/>
-      <c r="AL16" s="17"/>
-      <c r="AM16" s="17"/>
-      <c r="AN16" s="17"/>
-      <c r="AO16" s="17"/>
-      <c r="AP16" s="17"/>
-      <c r="AQ16" s="17"/>
-      <c r="AR16" s="17"/>
-      <c r="AS16" s="17"/>
-      <c r="AT16" s="17"/>
-      <c r="AU16" s="64"/>
-      <c r="AV16" s="64"/>
-      <c r="AW16" s="64"/>
-      <c r="AX16" s="64"/>
-      <c r="AY16" s="64"/>
-      <c r="AZ16" s="64"/>
-      <c r="BA16" s="64"/>
-      <c r="BB16" s="64"/>
-      <c r="BC16" s="64"/>
-      <c r="BD16" s="64"/>
-      <c r="BE16" s="64"/>
-      <c r="BF16" s="65"/>
-      <c r="BG16" s="17"/>
-      <c r="BH16" s="17"/>
-      <c r="BI16" s="17"/>
-      <c r="BJ16" s="17"/>
-      <c r="BK16" s="17"/>
-      <c r="BL16" s="17"/>
-      <c r="BM16" s="17"/>
-      <c r="BN16" s="17"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="16"/>
+      <c r="W16" s="16"/>
+      <c r="X16" s="16"/>
+      <c r="Y16" s="16"/>
+      <c r="Z16" s="16"/>
+      <c r="AA16" s="16"/>
+      <c r="AB16" s="16"/>
+      <c r="AC16" s="16"/>
+      <c r="AD16" s="16"/>
+      <c r="AE16" s="16"/>
+      <c r="AF16" s="16"/>
+      <c r="AG16" s="16"/>
+      <c r="AH16" s="16"/>
+      <c r="AI16" s="16"/>
+      <c r="AJ16" s="16"/>
+      <c r="AK16" s="16"/>
+      <c r="AL16" s="16"/>
+      <c r="AM16" s="16"/>
+      <c r="AN16" s="16"/>
+      <c r="AO16" s="16"/>
+      <c r="AP16" s="16"/>
+      <c r="AQ16" s="16"/>
+      <c r="AR16" s="16"/>
+      <c r="AS16" s="16"/>
+      <c r="AT16" s="16"/>
+      <c r="AU16" s="16"/>
+      <c r="AV16" s="16"/>
+      <c r="AW16" s="16"/>
+      <c r="AX16" s="16"/>
+      <c r="AY16" s="16"/>
+      <c r="AZ16" s="16"/>
+      <c r="BA16" s="16"/>
+      <c r="BB16" s="16"/>
+      <c r="BC16" s="16"/>
+      <c r="BD16" s="16"/>
+      <c r="BE16" s="16"/>
+      <c r="BF16" s="63"/>
+      <c r="BG16" s="16"/>
+      <c r="BH16" s="16"/>
+      <c r="BI16" s="16"/>
+      <c r="BJ16" s="16"/>
+      <c r="BK16" s="16"/>
+      <c r="BL16" s="16"/>
+      <c r="BM16" s="16"/>
+      <c r="BN16" s="16"/>
     </row>
     <row r="17" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-      <c r="U17" s="17"/>
-      <c r="V17" s="17"/>
-      <c r="W17" s="17"/>
-      <c r="X17" s="17"/>
-      <c r="Y17" s="17"/>
-      <c r="Z17" s="17"/>
-      <c r="AA17" s="17"/>
-      <c r="AB17" s="17"/>
-      <c r="AC17" s="17"/>
-      <c r="AD17" s="17"/>
-      <c r="AE17" s="17"/>
-      <c r="AF17" s="17"/>
-      <c r="AG17" s="17"/>
-      <c r="AH17" s="17"/>
-      <c r="AI17" s="17"/>
-      <c r="AJ17" s="17"/>
-      <c r="AK17" s="17"/>
-      <c r="AL17" s="17"/>
-      <c r="AM17" s="17"/>
-      <c r="AN17" s="17"/>
-      <c r="AO17" s="17"/>
-      <c r="AP17" s="17"/>
-      <c r="AQ17" s="17"/>
-      <c r="AR17" s="17"/>
-      <c r="AS17" s="17"/>
-      <c r="AT17" s="17"/>
-      <c r="AU17" s="64"/>
-      <c r="AV17" s="64"/>
-      <c r="AW17" s="64"/>
-      <c r="AX17" s="64"/>
-      <c r="AY17" s="64"/>
-      <c r="AZ17" s="64"/>
-      <c r="BA17" s="64"/>
-      <c r="BB17" s="64"/>
-      <c r="BC17" s="64"/>
-      <c r="BD17" s="64"/>
-      <c r="BE17" s="64"/>
-      <c r="BF17" s="65"/>
-      <c r="BG17" s="17"/>
-      <c r="BH17" s="17"/>
-      <c r="BI17" s="17"/>
-      <c r="BJ17" s="17"/>
-      <c r="BK17" s="17"/>
-      <c r="BL17" s="17"/>
-      <c r="BM17" s="17"/>
-      <c r="BN17" s="17"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="16"/>
+      <c r="T17" s="16"/>
+      <c r="U17" s="16"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="16"/>
+      <c r="X17" s="16"/>
+      <c r="Y17" s="16"/>
+      <c r="Z17" s="16"/>
+      <c r="AA17" s="16"/>
+      <c r="AB17" s="16"/>
+      <c r="AC17" s="16"/>
+      <c r="AD17" s="16"/>
+      <c r="AE17" s="16"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="16"/>
+      <c r="AH17" s="16"/>
+      <c r="AI17" s="16"/>
+      <c r="AJ17" s="16"/>
+      <c r="AK17" s="16"/>
+      <c r="AL17" s="16"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="16"/>
+      <c r="AO17" s="16"/>
+      <c r="AP17" s="16"/>
+      <c r="AQ17" s="16"/>
+      <c r="AR17" s="16"/>
+      <c r="AS17" s="16"/>
+      <c r="AT17" s="16"/>
+      <c r="AU17" s="16"/>
+      <c r="AV17" s="16"/>
+      <c r="AW17" s="16"/>
+      <c r="AX17" s="16"/>
+      <c r="AY17" s="16"/>
+      <c r="AZ17" s="16"/>
+      <c r="BA17" s="16"/>
+      <c r="BB17" s="16"/>
+      <c r="BC17" s="16"/>
+      <c r="BD17" s="16"/>
+      <c r="BE17" s="16"/>
+      <c r="BF17" s="63"/>
+      <c r="BG17" s="16"/>
+      <c r="BH17" s="16"/>
+      <c r="BI17" s="16"/>
+      <c r="BJ17" s="16"/>
+      <c r="BK17" s="16"/>
+      <c r="BL17" s="16"/>
+      <c r="BM17" s="16"/>
+      <c r="BN17" s="16"/>
     </row>
     <row r="18" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
-      <c r="U18" s="17"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="17"/>
-      <c r="X18" s="17"/>
-      <c r="Y18" s="17"/>
-      <c r="Z18" s="17"/>
-      <c r="AA18" s="17"/>
-      <c r="AB18" s="17"/>
-      <c r="AC18" s="17"/>
-      <c r="AD18" s="17"/>
-      <c r="AE18" s="17"/>
-      <c r="AF18" s="17"/>
-      <c r="AG18" s="17"/>
-      <c r="AH18" s="17"/>
-      <c r="AI18" s="17"/>
-      <c r="AJ18" s="17"/>
-      <c r="AK18" s="17"/>
-      <c r="AL18" s="17"/>
-      <c r="AM18" s="17"/>
-      <c r="AN18" s="17"/>
-      <c r="AO18" s="17"/>
-      <c r="AP18" s="17"/>
-      <c r="AQ18" s="17"/>
-      <c r="AR18" s="17"/>
-      <c r="AS18" s="17"/>
-      <c r="AT18" s="17"/>
-      <c r="AU18" s="64"/>
-      <c r="AV18" s="64"/>
-      <c r="AW18" s="64"/>
-      <c r="AX18" s="64"/>
-      <c r="AY18" s="64"/>
-      <c r="AZ18" s="64"/>
-      <c r="BA18" s="64"/>
-      <c r="BB18" s="64"/>
-      <c r="BC18" s="64"/>
-      <c r="BD18" s="64"/>
-      <c r="BE18" s="64"/>
-      <c r="BF18" s="65"/>
-      <c r="BG18" s="17"/>
-      <c r="BH18" s="17"/>
-      <c r="BI18" s="17"/>
-      <c r="BJ18" s="17"/>
-      <c r="BK18" s="17"/>
-      <c r="BL18" s="17"/>
-      <c r="BM18" s="17"/>
-      <c r="BN18" s="17"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="16"/>
+      <c r="X18" s="16"/>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="16"/>
+      <c r="AA18" s="16"/>
+      <c r="AB18" s="16"/>
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
+      <c r="AI18" s="16"/>
+      <c r="AJ18" s="16"/>
+      <c r="AK18" s="16"/>
+      <c r="AL18" s="16"/>
+      <c r="AM18" s="16"/>
+      <c r="AN18" s="16"/>
+      <c r="AO18" s="16"/>
+      <c r="AP18" s="16"/>
+      <c r="AQ18" s="16"/>
+      <c r="AR18" s="16"/>
+      <c r="AS18" s="16"/>
+      <c r="AT18" s="16"/>
+      <c r="AU18" s="16"/>
+      <c r="AV18" s="16"/>
+      <c r="AW18" s="16"/>
+      <c r="AX18" s="16"/>
+      <c r="AY18" s="16"/>
+      <c r="AZ18" s="16"/>
+      <c r="BA18" s="16"/>
+      <c r="BB18" s="16"/>
+      <c r="BC18" s="16"/>
+      <c r="BD18" s="16"/>
+      <c r="BE18" s="16"/>
+      <c r="BF18" s="63"/>
+      <c r="BG18" s="16"/>
+      <c r="BH18" s="16"/>
+      <c r="BI18" s="16"/>
+      <c r="BJ18" s="16"/>
+      <c r="BK18" s="16"/>
+      <c r="BL18" s="16"/>
+      <c r="BM18" s="16"/>
+      <c r="BN18" s="16"/>
     </row>
     <row r="19" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="17"/>
-      <c r="U19" s="17"/>
-      <c r="V19" s="17"/>
-      <c r="W19" s="17"/>
-      <c r="X19" s="17"/>
-      <c r="Y19" s="17"/>
-      <c r="Z19" s="17"/>
-      <c r="AA19" s="17"/>
-      <c r="AB19" s="17"/>
-      <c r="AC19" s="17"/>
-      <c r="AD19" s="17"/>
-      <c r="AE19" s="17"/>
-      <c r="AF19" s="17"/>
-      <c r="AG19" s="17"/>
-      <c r="AH19" s="17"/>
-      <c r="AI19" s="17"/>
-      <c r="AJ19" s="17"/>
-      <c r="AK19" s="17"/>
-      <c r="AL19" s="17"/>
-      <c r="AM19" s="17"/>
-      <c r="AN19" s="17"/>
-      <c r="AO19" s="17"/>
-      <c r="AP19" s="17"/>
-      <c r="AQ19" s="17"/>
-      <c r="AR19" s="17"/>
-      <c r="AS19" s="17"/>
-      <c r="AT19" s="17"/>
-      <c r="AU19" s="64"/>
-      <c r="AV19" s="64"/>
-      <c r="AW19" s="64"/>
-      <c r="AX19" s="64"/>
-      <c r="AY19" s="64"/>
-      <c r="AZ19" s="64"/>
-      <c r="BA19" s="64"/>
-      <c r="BB19" s="64"/>
-      <c r="BC19" s="64"/>
-      <c r="BD19" s="64"/>
-      <c r="BE19" s="64"/>
-      <c r="BF19" s="65"/>
-      <c r="BG19" s="17"/>
-      <c r="BH19" s="17"/>
-      <c r="BI19" s="17"/>
-      <c r="BJ19" s="17"/>
-      <c r="BK19" s="17"/>
-      <c r="BL19" s="17"/>
-      <c r="BM19" s="17"/>
-      <c r="BN19" s="17"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="16"/>
+      <c r="X19" s="16"/>
+      <c r="Y19" s="16"/>
+      <c r="Z19" s="16"/>
+      <c r="AA19" s="16"/>
+      <c r="AB19" s="16"/>
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="16"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+      <c r="AI19" s="16"/>
+      <c r="AJ19" s="16"/>
+      <c r="AK19" s="16"/>
+      <c r="AL19" s="16"/>
+      <c r="AM19" s="16"/>
+      <c r="AN19" s="16"/>
+      <c r="AO19" s="16"/>
+      <c r="AP19" s="16"/>
+      <c r="AQ19" s="16"/>
+      <c r="AR19" s="16"/>
+      <c r="AS19" s="16"/>
+      <c r="AT19" s="16"/>
+      <c r="AU19" s="16"/>
+      <c r="AV19" s="16"/>
+      <c r="AW19" s="16"/>
+      <c r="AX19" s="16"/>
+      <c r="AY19" s="16"/>
+      <c r="AZ19" s="16"/>
+      <c r="BA19" s="16"/>
+      <c r="BB19" s="16"/>
+      <c r="BC19" s="16"/>
+      <c r="BD19" s="16"/>
+      <c r="BE19" s="16"/>
+      <c r="BF19" s="63"/>
+      <c r="BG19" s="16"/>
+      <c r="BH19" s="16"/>
+      <c r="BI19" s="16"/>
+      <c r="BJ19" s="16"/>
+      <c r="BK19" s="16"/>
+      <c r="BL19" s="16"/>
+      <c r="BM19" s="16"/>
+      <c r="BN19" s="16"/>
     </row>
     <row r="20" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="17"/>
-      <c r="U20" s="17"/>
-      <c r="V20" s="17"/>
-      <c r="W20" s="17"/>
-      <c r="X20" s="17"/>
-      <c r="Y20" s="17"/>
-      <c r="Z20" s="17"/>
-      <c r="AA20" s="17"/>
-      <c r="AB20" s="17"/>
-      <c r="AC20" s="17"/>
-      <c r="AD20" s="17"/>
-      <c r="AE20" s="17"/>
-      <c r="AF20" s="17"/>
-      <c r="AG20" s="17"/>
-      <c r="AH20" s="17"/>
-      <c r="AI20" s="17"/>
-      <c r="AJ20" s="17"/>
-      <c r="AK20" s="17"/>
-      <c r="AL20" s="17"/>
-      <c r="AM20" s="17"/>
-      <c r="AN20" s="17"/>
-      <c r="AO20" s="17"/>
-      <c r="AP20" s="17"/>
-      <c r="AQ20" s="17"/>
-      <c r="AR20" s="17"/>
-      <c r="AS20" s="17"/>
-      <c r="AT20" s="17"/>
-      <c r="AU20" s="64"/>
-      <c r="AV20" s="64"/>
-      <c r="AW20" s="64"/>
-      <c r="AX20" s="64"/>
-      <c r="AY20" s="64"/>
-      <c r="AZ20" s="64"/>
-      <c r="BA20" s="64"/>
-      <c r="BB20" s="64"/>
-      <c r="BC20" s="64"/>
-      <c r="BD20" s="64"/>
-      <c r="BE20" s="64"/>
-      <c r="BF20" s="65"/>
-      <c r="BG20" s="17"/>
-      <c r="BH20" s="17"/>
-      <c r="BI20" s="17"/>
-      <c r="BJ20" s="17"/>
-      <c r="BK20" s="17"/>
-      <c r="BL20" s="17"/>
-      <c r="BM20" s="17"/>
-      <c r="BN20" s="17"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="16"/>
+      <c r="X20" s="16"/>
+      <c r="Y20" s="16"/>
+      <c r="Z20" s="16"/>
+      <c r="AA20" s="16"/>
+      <c r="AB20" s="16"/>
+      <c r="AC20" s="16"/>
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="16"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
+      <c r="AI20" s="16"/>
+      <c r="AJ20" s="16"/>
+      <c r="AK20" s="16"/>
+      <c r="AL20" s="16"/>
+      <c r="AM20" s="16"/>
+      <c r="AN20" s="16"/>
+      <c r="AO20" s="16"/>
+      <c r="AP20" s="16"/>
+      <c r="AQ20" s="16"/>
+      <c r="AR20" s="16"/>
+      <c r="AS20" s="16"/>
+      <c r="AT20" s="16"/>
+      <c r="AU20" s="16"/>
+      <c r="AV20" s="16"/>
+      <c r="AW20" s="16"/>
+      <c r="AX20" s="16"/>
+      <c r="AY20" s="16"/>
+      <c r="AZ20" s="16"/>
+      <c r="BA20" s="16"/>
+      <c r="BB20" s="16"/>
+      <c r="BC20" s="16"/>
+      <c r="BD20" s="16"/>
+      <c r="BE20" s="16"/>
+      <c r="BF20" s="63"/>
+      <c r="BG20" s="16"/>
+      <c r="BH20" s="16"/>
+      <c r="BI20" s="16"/>
+      <c r="BJ20" s="16"/>
+      <c r="BK20" s="16"/>
+      <c r="BL20" s="16"/>
+      <c r="BM20" s="16"/>
+      <c r="BN20" s="16"/>
     </row>
     <row r="21" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
-      <c r="U21" s="17"/>
-      <c r="V21" s="17"/>
-      <c r="W21" s="17"/>
-      <c r="X21" s="17"/>
-      <c r="Y21" s="17"/>
-      <c r="Z21" s="17"/>
-      <c r="AA21" s="17"/>
-      <c r="AB21" s="17"/>
-      <c r="AC21" s="17"/>
-      <c r="AD21" s="17"/>
-      <c r="AE21" s="17"/>
-      <c r="AF21" s="17"/>
-      <c r="AG21" s="17"/>
-      <c r="AH21" s="17"/>
-      <c r="AI21" s="17"/>
-      <c r="AJ21" s="17"/>
-      <c r="AK21" s="17"/>
-      <c r="AL21" s="17"/>
-      <c r="AM21" s="17"/>
-      <c r="AN21" s="17"/>
-      <c r="AO21" s="17"/>
-      <c r="AP21" s="17"/>
-      <c r="AQ21" s="17"/>
-      <c r="AR21" s="17"/>
-      <c r="AS21" s="17"/>
-      <c r="AT21" s="17"/>
-      <c r="AU21" s="64"/>
-      <c r="AV21" s="64"/>
-      <c r="AW21" s="64"/>
-      <c r="AX21" s="64"/>
-      <c r="AY21" s="64"/>
-      <c r="AZ21" s="64"/>
-      <c r="BA21" s="64"/>
-      <c r="BB21" s="64"/>
-      <c r="BC21" s="64"/>
-      <c r="BD21" s="64"/>
-      <c r="BE21" s="64"/>
-      <c r="BF21" s="65"/>
-      <c r="BG21" s="17"/>
-      <c r="BH21" s="17"/>
-      <c r="BI21" s="17"/>
-      <c r="BJ21" s="17"/>
-      <c r="BK21" s="17"/>
-      <c r="BL21" s="17"/>
-      <c r="BM21" s="17"/>
-      <c r="BN21" s="17"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="16"/>
+      <c r="X21" s="16"/>
+      <c r="Y21" s="16"/>
+      <c r="Z21" s="16"/>
+      <c r="AA21" s="16"/>
+      <c r="AB21" s="16"/>
+      <c r="AC21" s="16"/>
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="16"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="16"/>
+      <c r="AI21" s="16"/>
+      <c r="AJ21" s="16"/>
+      <c r="AK21" s="16"/>
+      <c r="AL21" s="16"/>
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="16"/>
+      <c r="AO21" s="16"/>
+      <c r="AP21" s="16"/>
+      <c r="AQ21" s="16"/>
+      <c r="AR21" s="16"/>
+      <c r="AS21" s="16"/>
+      <c r="AT21" s="16"/>
+      <c r="AU21" s="16"/>
+      <c r="AV21" s="16"/>
+      <c r="AW21" s="16"/>
+      <c r="AX21" s="16"/>
+      <c r="AY21" s="16"/>
+      <c r="AZ21" s="16"/>
+      <c r="BA21" s="16"/>
+      <c r="BB21" s="16"/>
+      <c r="BC21" s="16"/>
+      <c r="BD21" s="16"/>
+      <c r="BE21" s="16"/>
+      <c r="BF21" s="63"/>
+      <c r="BG21" s="16"/>
+      <c r="BH21" s="16"/>
+      <c r="BI21" s="16"/>
+      <c r="BJ21" s="16"/>
+      <c r="BK21" s="16"/>
+      <c r="BL21" s="16"/>
+      <c r="BM21" s="16"/>
+      <c r="BN21" s="16"/>
     </row>
     <row r="22" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="17"/>
-      <c r="U22" s="17"/>
-      <c r="V22" s="17"/>
-      <c r="W22" s="17"/>
-      <c r="X22" s="17"/>
-      <c r="Y22" s="17"/>
-      <c r="Z22" s="17"/>
-      <c r="AA22" s="17"/>
-      <c r="AB22" s="17"/>
-      <c r="AC22" s="17"/>
-      <c r="AD22" s="17"/>
-      <c r="AE22" s="17"/>
-      <c r="AF22" s="17"/>
-      <c r="AG22" s="17"/>
-      <c r="AH22" s="17"/>
-      <c r="AI22" s="17"/>
-      <c r="AJ22" s="17"/>
-      <c r="AK22" s="17"/>
-      <c r="AL22" s="17"/>
-      <c r="AM22" s="17"/>
-      <c r="AN22" s="17"/>
-      <c r="AO22" s="17"/>
-      <c r="AP22" s="17"/>
-      <c r="AQ22" s="17"/>
-      <c r="AR22" s="17"/>
-      <c r="AS22" s="17"/>
-      <c r="AT22" s="17"/>
-      <c r="AU22" s="64"/>
-      <c r="AV22" s="64"/>
-      <c r="AW22" s="64"/>
-      <c r="AX22" s="64"/>
-      <c r="AY22" s="64"/>
-      <c r="AZ22" s="64"/>
-      <c r="BA22" s="64"/>
-      <c r="BB22" s="64"/>
-      <c r="BC22" s="64"/>
-      <c r="BD22" s="64"/>
-      <c r="BE22" s="64"/>
-      <c r="BF22" s="65"/>
-      <c r="BG22" s="17"/>
-      <c r="BH22" s="17"/>
-      <c r="BI22" s="17"/>
-      <c r="BJ22" s="17"/>
-      <c r="BK22" s="17"/>
-      <c r="BL22" s="17"/>
-      <c r="BM22" s="17"/>
-      <c r="BN22" s="17"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="16"/>
+      <c r="T22" s="16"/>
+      <c r="U22" s="16"/>
+      <c r="V22" s="16"/>
+      <c r="W22" s="16"/>
+      <c r="X22" s="16"/>
+      <c r="Y22" s="16"/>
+      <c r="Z22" s="16"/>
+      <c r="AA22" s="16"/>
+      <c r="AB22" s="16"/>
+      <c r="AC22" s="16"/>
+      <c r="AD22" s="16"/>
+      <c r="AE22" s="16"/>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16"/>
+      <c r="AH22" s="16"/>
+      <c r="AI22" s="16"/>
+      <c r="AJ22" s="16"/>
+      <c r="AK22" s="16"/>
+      <c r="AL22" s="16"/>
+      <c r="AM22" s="16"/>
+      <c r="AN22" s="16"/>
+      <c r="AO22" s="16"/>
+      <c r="AP22" s="16"/>
+      <c r="AQ22" s="16"/>
+      <c r="AR22" s="16"/>
+      <c r="AS22" s="16"/>
+      <c r="AT22" s="16"/>
+      <c r="AU22" s="16"/>
+      <c r="AV22" s="16"/>
+      <c r="AW22" s="16"/>
+      <c r="AX22" s="16"/>
+      <c r="AY22" s="16"/>
+      <c r="AZ22" s="16"/>
+      <c r="BA22" s="16"/>
+      <c r="BB22" s="16"/>
+      <c r="BC22" s="16"/>
+      <c r="BD22" s="16"/>
+      <c r="BE22" s="16"/>
+      <c r="BF22" s="63"/>
+      <c r="BG22" s="16"/>
+      <c r="BH22" s="16"/>
+      <c r="BI22" s="16"/>
+      <c r="BJ22" s="16"/>
+      <c r="BK22" s="16"/>
+      <c r="BL22" s="16"/>
+      <c r="BM22" s="16"/>
+      <c r="BN22" s="16"/>
     </row>
     <row r="23" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="17"/>
-      <c r="R23" s="17"/>
-      <c r="S23" s="17"/>
-      <c r="T23" s="17"/>
-      <c r="U23" s="17"/>
-      <c r="V23" s="17"/>
-      <c r="W23" s="17"/>
-      <c r="X23" s="17"/>
-      <c r="Y23" s="17"/>
-      <c r="Z23" s="17"/>
-      <c r="AA23" s="17"/>
-      <c r="AB23" s="17"/>
-      <c r="AC23" s="17"/>
-      <c r="AD23" s="17"/>
-      <c r="AE23" s="17"/>
-      <c r="AF23" s="17"/>
-      <c r="AG23" s="17"/>
-      <c r="AH23" s="17"/>
-      <c r="AI23" s="17"/>
-      <c r="AJ23" s="17"/>
-      <c r="AK23" s="17"/>
-      <c r="AL23" s="17"/>
-      <c r="AM23" s="17"/>
-      <c r="AN23" s="17"/>
-      <c r="AO23" s="17"/>
-      <c r="AP23" s="17"/>
-      <c r="AQ23" s="17"/>
-      <c r="AR23" s="17"/>
-      <c r="AS23" s="17"/>
-      <c r="AT23" s="17"/>
-      <c r="AU23" s="64"/>
-      <c r="AV23" s="64"/>
-      <c r="AW23" s="64"/>
-      <c r="AX23" s="64"/>
-      <c r="AY23" s="64"/>
-      <c r="AZ23" s="64"/>
-      <c r="BA23" s="64"/>
-      <c r="BB23" s="64"/>
-      <c r="BC23" s="64"/>
-      <c r="BD23" s="64"/>
-      <c r="BE23" s="64"/>
-      <c r="BF23" s="65"/>
-      <c r="BG23" s="17"/>
-      <c r="BH23" s="17"/>
-      <c r="BI23" s="17"/>
-      <c r="BJ23" s="17"/>
-      <c r="BK23" s="17"/>
-      <c r="BL23" s="17"/>
-      <c r="BM23" s="17"/>
-      <c r="BN23" s="17"/>
-    </row>
-    <row r="24" spans="1:96" s="16" customFormat="1" ht="10.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="16"/>
+      <c r="T23" s="16"/>
+      <c r="U23" s="16"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="16"/>
+      <c r="X23" s="16"/>
+      <c r="Y23" s="16"/>
+      <c r="Z23" s="16"/>
+      <c r="AA23" s="16"/>
+      <c r="AB23" s="16"/>
+      <c r="AC23" s="16"/>
+      <c r="AD23" s="16"/>
+      <c r="AE23" s="16"/>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16"/>
+      <c r="AH23" s="16"/>
+      <c r="AI23" s="16"/>
+      <c r="AJ23" s="16"/>
+      <c r="AK23" s="16"/>
+      <c r="AL23" s="16"/>
+      <c r="AM23" s="16"/>
+      <c r="AN23" s="16"/>
+      <c r="AO23" s="16"/>
+      <c r="AP23" s="16"/>
+      <c r="AQ23" s="16"/>
+      <c r="AR23" s="16"/>
+      <c r="AS23" s="16"/>
+      <c r="AT23" s="16"/>
+      <c r="AU23" s="16"/>
+      <c r="AV23" s="16"/>
+      <c r="AW23" s="16"/>
+      <c r="AX23" s="16"/>
+      <c r="AY23" s="16"/>
+      <c r="AZ23" s="16"/>
+      <c r="BA23" s="16"/>
+      <c r="BB23" s="16"/>
+      <c r="BC23" s="16"/>
+      <c r="BD23" s="16"/>
+      <c r="BE23" s="16"/>
+      <c r="BF23" s="63"/>
+      <c r="BG23" s="16"/>
+      <c r="BH23" s="16"/>
+      <c r="BI23" s="16"/>
+      <c r="BJ23" s="16"/>
+      <c r="BK23" s="16"/>
+      <c r="BL23" s="16"/>
+      <c r="BM23" s="16"/>
+      <c r="BN23" s="16"/>
+    </row>
+    <row r="24" spans="1:96" s="15" customFormat="1" ht="10.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="18"/>
-      <c r="P24" s="18"/>
-      <c r="Q24" s="18"/>
-      <c r="R24" s="18"/>
-      <c r="S24" s="18"/>
-      <c r="T24" s="18"/>
-      <c r="U24" s="18"/>
-      <c r="V24" s="18"/>
-      <c r="W24" s="18"/>
-      <c r="X24" s="18"/>
-      <c r="Y24" s="18"/>
-      <c r="Z24" s="18"/>
-      <c r="AA24" s="18"/>
-      <c r="AB24" s="18"/>
-      <c r="AC24" s="18"/>
-      <c r="AD24" s="18"/>
-      <c r="AE24" s="18"/>
-      <c r="AF24" s="18"/>
-      <c r="AG24" s="18"/>
-      <c r="AH24" s="18"/>
-      <c r="AI24" s="18"/>
-      <c r="AJ24" s="18"/>
-      <c r="AK24" s="18"/>
-      <c r="AL24" s="18"/>
-      <c r="AM24" s="18"/>
-      <c r="AN24" s="18"/>
-      <c r="AO24" s="18"/>
-      <c r="AP24" s="18"/>
-      <c r="AQ24" s="18"/>
-      <c r="AR24" s="18"/>
-      <c r="AS24" s="18"/>
-      <c r="AT24" s="18"/>
-      <c r="AU24" s="18"/>
-      <c r="AV24" s="18"/>
-      <c r="AW24" s="18"/>
-      <c r="AX24" s="18"/>
-      <c r="AY24" s="18"/>
-      <c r="AZ24" s="18"/>
-      <c r="BA24" s="18"/>
-      <c r="BB24" s="18"/>
-      <c r="BC24" s="18"/>
-      <c r="BD24" s="18"/>
-      <c r="BE24" s="18"/>
-      <c r="BF24" s="66"/>
-      <c r="BG24" s="18"/>
-      <c r="BH24" s="18"/>
-      <c r="BI24" s="18"/>
-      <c r="BJ24" s="18"/>
-      <c r="BK24" s="18"/>
-      <c r="BL24" s="18"/>
-      <c r="BM24" s="18"/>
-      <c r="BN24" s="18"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
+      <c r="U24" s="17"/>
+      <c r="V24" s="17"/>
+      <c r="W24" s="17"/>
+      <c r="X24" s="17"/>
+      <c r="Y24" s="17"/>
+      <c r="Z24" s="17"/>
+      <c r="AA24" s="17"/>
+      <c r="AB24" s="17"/>
+      <c r="AC24" s="17"/>
+      <c r="AD24" s="17"/>
+      <c r="AE24" s="17"/>
+      <c r="AF24" s="17"/>
+      <c r="AG24" s="17"/>
+      <c r="AH24" s="17"/>
+      <c r="AI24" s="17"/>
+      <c r="AJ24" s="17"/>
+      <c r="AK24" s="17"/>
+      <c r="AL24" s="17"/>
+      <c r="AM24" s="17"/>
+      <c r="AN24" s="17"/>
+      <c r="AO24" s="17"/>
+      <c r="AP24" s="17"/>
+      <c r="AQ24" s="17"/>
+      <c r="AR24" s="17"/>
+      <c r="AS24" s="17"/>
+      <c r="AT24" s="17"/>
+      <c r="AU24" s="17"/>
+      <c r="AV24" s="17"/>
+      <c r="AW24" s="17"/>
+      <c r="AX24" s="17"/>
+      <c r="AY24" s="17"/>
+      <c r="AZ24" s="17"/>
+      <c r="BA24" s="17"/>
+      <c r="BB24" s="17"/>
+      <c r="BC24" s="17"/>
+      <c r="BD24" s="17"/>
+      <c r="BE24" s="17"/>
+      <c r="BF24" s="64"/>
+      <c r="BG24" s="17"/>
+      <c r="BH24" s="17"/>
+      <c r="BI24" s="17"/>
+      <c r="BJ24" s="17"/>
+      <c r="BK24" s="17"/>
+      <c r="BL24" s="17"/>
+      <c r="BM24" s="17"/>
+      <c r="BN24" s="17"/>
       <c r="BO24"/>
       <c r="BP24"/>
       <c r="BQ24"/>
@@ -5895,1340 +5865,524 @@
       <c r="CR24"/>
     </row>
     <row r="25" spans="1:96" ht="7.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="17"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
-      <c r="O25" s="17"/>
-      <c r="P25" s="17"/>
-      <c r="Q25" s="17"/>
-      <c r="R25" s="17"/>
-      <c r="S25" s="17"/>
-      <c r="T25" s="17"/>
-      <c r="U25" s="17"/>
-      <c r="V25" s="17"/>
-      <c r="W25" s="17"/>
-      <c r="X25" s="17"/>
-      <c r="Y25" s="17"/>
-      <c r="Z25" s="17"/>
-      <c r="AA25" s="17"/>
-      <c r="AB25" s="17"/>
-      <c r="AC25" s="17"/>
-      <c r="AD25" s="17"/>
-      <c r="AE25" s="17"/>
-      <c r="AF25" s="17"/>
-      <c r="AG25" s="17"/>
-      <c r="AH25" s="17"/>
-      <c r="AI25" s="17"/>
-      <c r="AJ25" s="17"/>
-      <c r="AK25" s="17"/>
-      <c r="AL25" s="17"/>
-      <c r="AM25" s="17"/>
-      <c r="AN25" s="17"/>
-      <c r="AO25" s="17"/>
-      <c r="AP25" s="17"/>
-      <c r="AQ25" s="17"/>
-      <c r="AR25" s="17"/>
-      <c r="AS25" s="17"/>
-      <c r="AT25" s="17"/>
-      <c r="AU25" s="64"/>
-      <c r="AV25" s="64"/>
-      <c r="AW25" s="64"/>
-      <c r="AX25" s="64"/>
-      <c r="AY25" s="64"/>
-      <c r="AZ25" s="64"/>
-      <c r="BA25" s="64"/>
-      <c r="BB25" s="64"/>
-      <c r="BC25" s="64"/>
-      <c r="BD25" s="64"/>
-      <c r="BE25" s="64"/>
-      <c r="BF25" s="65"/>
-      <c r="BG25" s="17"/>
-      <c r="BH25" s="17"/>
-      <c r="BI25" s="17"/>
-      <c r="BJ25" s="17"/>
-      <c r="BK25" s="17"/>
-      <c r="BL25" s="17"/>
-      <c r="BM25" s="17"/>
-      <c r="BN25" s="17"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="16"/>
+      <c r="U25" s="16"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="16"/>
+      <c r="X25" s="16"/>
+      <c r="Y25" s="16"/>
+      <c r="Z25" s="16"/>
+      <c r="AA25" s="16"/>
+      <c r="AB25" s="16"/>
+      <c r="AC25" s="16"/>
+      <c r="AD25" s="16"/>
+      <c r="AE25" s="16"/>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="16"/>
+      <c r="AH25" s="16"/>
+      <c r="AI25" s="16"/>
+      <c r="AJ25" s="16"/>
+      <c r="AK25" s="16"/>
+      <c r="AL25" s="16"/>
+      <c r="AM25" s="16"/>
+      <c r="AN25" s="16"/>
+      <c r="AO25" s="16"/>
+      <c r="AP25" s="16"/>
+      <c r="AQ25" s="16"/>
+      <c r="AR25" s="16"/>
+      <c r="AS25" s="16"/>
+      <c r="AT25" s="16"/>
+      <c r="AU25" s="16"/>
+      <c r="AV25" s="16"/>
+      <c r="AW25" s="16"/>
+      <c r="AX25" s="16"/>
+      <c r="AY25" s="16"/>
+      <c r="AZ25" s="16"/>
+      <c r="BA25" s="16"/>
+      <c r="BB25" s="16"/>
+      <c r="BC25" s="16"/>
+      <c r="BD25" s="16"/>
+      <c r="BE25" s="16"/>
+      <c r="BF25" s="63"/>
+      <c r="BG25" s="16"/>
+      <c r="BH25" s="16"/>
+      <c r="BI25" s="16"/>
+      <c r="BJ25" s="16"/>
+      <c r="BK25" s="16"/>
+      <c r="BL25" s="16"/>
+      <c r="BM25" s="16"/>
+      <c r="BN25" s="16"/>
     </row>
     <row r="26" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="W26" s="26"/>
-      <c r="X26" s="27"/>
-      <c r="Y26" s="28"/>
-      <c r="AU26" s="4"/>
-      <c r="AV26" s="4"/>
-      <c r="AW26" s="4"/>
-      <c r="AX26" s="4"/>
-      <c r="AY26" s="4"/>
-      <c r="AZ26" s="4"/>
-      <c r="BA26" s="4"/>
-      <c r="BB26" s="4"/>
-      <c r="BC26" s="4"/>
-      <c r="BD26" s="4"/>
-      <c r="BE26" s="4"/>
-      <c r="BF26" s="67"/>
+      <c r="W26" s="25"/>
+      <c r="X26" s="26"/>
+      <c r="Y26" s="27"/>
+      <c r="BF26" s="65"/>
     </row>
     <row r="27" spans="1:96" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="24"/>
-      <c r="R27" s="34"/>
-      <c r="W27" s="29"/>
-      <c r="X27" s="4"/>
-      <c r="Y27" s="30"/>
-      <c r="AF27" s="34"/>
-      <c r="AU27" s="68"/>
-      <c r="AV27" s="4"/>
-      <c r="AW27" s="4"/>
-      <c r="AX27" s="4"/>
-      <c r="AY27" s="4"/>
-      <c r="AZ27" s="4"/>
-      <c r="BA27" s="4"/>
-      <c r="BB27" s="4"/>
-      <c r="BC27" s="4"/>
-      <c r="BD27" s="4"/>
-      <c r="BE27" s="4"/>
-      <c r="BF27" s="67"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="23"/>
+      <c r="R27" s="33"/>
+      <c r="W27" s="28"/>
+      <c r="Y27" s="29"/>
+      <c r="AF27" s="33"/>
+      <c r="AU27" s="33"/>
+      <c r="BF27" s="65"/>
     </row>
     <row r="28" spans="1:96" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="25"/>
-      <c r="W28" s="31"/>
-      <c r="X28" s="32"/>
-      <c r="Y28" s="33"/>
-      <c r="AU28" s="4"/>
-      <c r="AV28" s="4"/>
-      <c r="AW28" s="4"/>
-      <c r="AX28" s="4"/>
-      <c r="AY28" s="4"/>
-      <c r="AZ28" s="4"/>
-      <c r="BA28" s="4"/>
-      <c r="BB28" s="4"/>
-      <c r="BC28" s="4"/>
-      <c r="BD28" s="4"/>
-      <c r="BE28" s="4"/>
-      <c r="BF28" s="67"/>
+      <c r="M28" s="24"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="31"/>
+      <c r="Y28" s="32"/>
+      <c r="BF28" s="65"/>
     </row>
     <row r="29" spans="1:96" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="W29" s="26"/>
-      <c r="X29" s="27"/>
-      <c r="Y29" s="28"/>
-      <c r="AB29" s="35"/>
-      <c r="AC29" s="35"/>
-      <c r="AD29" s="35"/>
-      <c r="AE29" s="35"/>
-      <c r="AF29" s="35"/>
-      <c r="AG29" s="35"/>
-      <c r="AH29" s="35"/>
-      <c r="AI29" s="35"/>
-      <c r="AJ29" s="35"/>
-      <c r="AK29" s="35"/>
-      <c r="AM29" s="22"/>
-      <c r="AN29" s="20"/>
-      <c r="AO29" s="21"/>
-      <c r="AQ29" s="35"/>
-      <c r="AR29" s="35"/>
-      <c r="AS29" s="35"/>
-      <c r="AT29" s="35"/>
-      <c r="AU29" s="35"/>
-      <c r="AV29" s="35"/>
-      <c r="AW29" s="35"/>
-      <c r="AX29" s="35"/>
-      <c r="AY29" s="37"/>
-      <c r="AZ29" s="37"/>
-      <c r="BA29" s="4"/>
-      <c r="BB29" s="22"/>
-      <c r="BC29" s="20"/>
-      <c r="BD29" s="4"/>
-      <c r="BE29" s="4"/>
-      <c r="BF29" s="67"/>
-      <c r="BJ29" s="22"/>
-      <c r="BK29" s="19"/>
-      <c r="BL29" s="19"/>
-      <c r="BM29" s="19"/>
-      <c r="BN29" s="19"/>
+      <c r="W29" s="25"/>
+      <c r="X29" s="26"/>
+      <c r="Y29" s="27"/>
+      <c r="AB29" s="34"/>
+      <c r="AC29" s="34"/>
+      <c r="AD29" s="34"/>
+      <c r="AE29" s="34"/>
+      <c r="AF29" s="34"/>
+      <c r="AG29" s="34"/>
+      <c r="AH29" s="34"/>
+      <c r="AI29" s="34"/>
+      <c r="AJ29" s="34"/>
+      <c r="AK29" s="34"/>
+      <c r="AM29" s="21"/>
+      <c r="AN29" s="19"/>
+      <c r="AO29" s="20"/>
+      <c r="AQ29" s="34"/>
+      <c r="AR29" s="34"/>
+      <c r="AS29" s="34"/>
+      <c r="AT29" s="34"/>
+      <c r="AU29" s="34"/>
+      <c r="AV29" s="34"/>
+      <c r="AW29" s="34"/>
+      <c r="AX29" s="34"/>
+      <c r="AY29" s="36"/>
+      <c r="AZ29" s="36"/>
+      <c r="BB29" s="21"/>
+      <c r="BC29" s="19"/>
+      <c r="BF29" s="65"/>
+      <c r="BJ29" s="21"/>
+      <c r="BK29" s="18"/>
+      <c r="BL29" s="18"/>
+      <c r="BM29" s="18"/>
+      <c r="BN29" s="18"/>
     </row>
     <row r="30" spans="1:96" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19"/>
-      <c r="P30" s="19"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="19"/>
-      <c r="S30" s="19"/>
-      <c r="T30" s="19"/>
-      <c r="U30" s="19"/>
-      <c r="V30" s="20"/>
-      <c r="W30" s="21"/>
-      <c r="X30" s="6"/>
-      <c r="Y30" s="7"/>
-      <c r="Z30" s="22"/>
-      <c r="AA30" s="19"/>
-      <c r="AB30" s="36"/>
-      <c r="AC30" s="36"/>
-      <c r="AD30" s="36"/>
-      <c r="AE30" s="36"/>
-      <c r="AF30" s="36"/>
-      <c r="AG30" s="36"/>
-      <c r="AH30" s="36"/>
-      <c r="AI30" s="36"/>
-      <c r="AJ30" s="36"/>
-      <c r="AK30" s="36"/>
-      <c r="AL30" s="19"/>
-      <c r="AP30" s="19"/>
-      <c r="AQ30" s="36"/>
-      <c r="AR30" s="36"/>
-      <c r="AS30" s="36"/>
-      <c r="AT30" s="36"/>
-      <c r="AU30" s="36"/>
-      <c r="AV30" s="36"/>
-      <c r="AW30" s="36"/>
-      <c r="AX30" s="36"/>
-      <c r="AY30" s="36"/>
-      <c r="AZ30" s="36"/>
-      <c r="BA30" s="19"/>
-      <c r="BB30" s="4"/>
-      <c r="BC30" s="5"/>
-      <c r="BD30" s="4"/>
-      <c r="BE30" s="4"/>
-      <c r="BF30" s="67"/>
-      <c r="BJ30" s="38"/>
-      <c r="BK30" s="4"/>
-      <c r="BL30" s="4"/>
-      <c r="BM30" s="4"/>
-      <c r="BN30" s="4"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="19"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="19"/>
+      <c r="W30" s="20"/>
+      <c r="X30" s="5"/>
+      <c r="Y30" s="6"/>
+      <c r="Z30" s="21"/>
+      <c r="AA30" s="18"/>
+      <c r="AB30" s="35"/>
+      <c r="AC30" s="35"/>
+      <c r="AD30" s="35"/>
+      <c r="AE30" s="35"/>
+      <c r="AF30" s="35"/>
+      <c r="AG30" s="35"/>
+      <c r="AH30" s="35"/>
+      <c r="AI30" s="35"/>
+      <c r="AJ30" s="35"/>
+      <c r="AK30" s="35"/>
+      <c r="AL30" s="18"/>
+      <c r="AP30" s="18"/>
+      <c r="AQ30" s="35"/>
+      <c r="AR30" s="35"/>
+      <c r="AS30" s="35"/>
+      <c r="AT30" s="35"/>
+      <c r="AU30" s="35"/>
+      <c r="AV30" s="35"/>
+      <c r="AW30" s="35"/>
+      <c r="AX30" s="35"/>
+      <c r="AY30" s="35"/>
+      <c r="AZ30" s="35"/>
+      <c r="BA30" s="18"/>
+      <c r="BC30" s="4"/>
+      <c r="BF30" s="65"/>
+      <c r="BJ30" s="37"/>
     </row>
     <row r="31" spans="1:96" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
-      <c r="M31" s="5"/>
-      <c r="AU31" s="4"/>
-      <c r="AV31" s="4"/>
-      <c r="AW31" s="4"/>
-      <c r="AX31" s="4"/>
-      <c r="AY31" s="4"/>
-      <c r="AZ31" s="4"/>
-      <c r="BA31" s="4"/>
-      <c r="BB31" s="4"/>
-      <c r="BC31" s="5"/>
-      <c r="BD31" s="4"/>
-      <c r="BE31" s="4"/>
-      <c r="BF31" s="67"/>
-      <c r="BJ31" s="38"/>
-      <c r="BK31" s="4"/>
-      <c r="BL31" s="4"/>
-      <c r="BM31" s="4"/>
-      <c r="BN31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="BC31" s="4"/>
+      <c r="BF31" s="65"/>
+      <c r="BJ31" s="37"/>
     </row>
     <row r="32" spans="1:96" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="5"/>
+      <c r="M32" s="4"/>
       <c r="W32" t="s">
         <v>88</v>
       </c>
-      <c r="AU32" s="4"/>
-      <c r="AV32" s="4"/>
-      <c r="AW32" s="4"/>
-      <c r="AX32" s="4"/>
-      <c r="AY32" s="4"/>
-      <c r="AZ32" s="4"/>
-      <c r="BA32" s="4"/>
-      <c r="BB32" s="4"/>
-      <c r="BC32" s="5"/>
-      <c r="BD32" s="4"/>
-      <c r="BE32" s="4"/>
-      <c r="BF32" s="67"/>
-      <c r="BJ32" s="38"/>
-      <c r="BK32" s="4"/>
-      <c r="BL32" s="4"/>
-      <c r="BM32" s="4"/>
-      <c r="BN32" s="4"/>
-    </row>
-    <row r="33" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="5"/>
-      <c r="AU33" s="4"/>
-      <c r="AV33" s="4"/>
-      <c r="AW33" s="4"/>
-      <c r="AX33" s="4"/>
-      <c r="AY33" s="4"/>
-      <c r="AZ33" s="4"/>
-      <c r="BA33" s="4"/>
-      <c r="BB33" s="4"/>
-      <c r="BC33" s="5"/>
-      <c r="BD33" s="4"/>
-      <c r="BE33" s="4"/>
-      <c r="BF33" s="67"/>
-      <c r="BJ33" s="38"/>
-      <c r="BK33" s="4"/>
-      <c r="BL33" s="4"/>
-      <c r="BM33" s="4"/>
-      <c r="BN33" s="4"/>
-    </row>
-    <row r="34" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="5"/>
-      <c r="AU34" s="4"/>
-      <c r="AV34" s="4"/>
-      <c r="AW34" s="4"/>
-      <c r="AX34" s="4"/>
-      <c r="AY34" s="4"/>
-      <c r="AZ34" s="4"/>
-      <c r="BA34" s="4"/>
-      <c r="BB34" s="4"/>
-      <c r="BC34" s="5"/>
-      <c r="BD34" s="4"/>
-      <c r="BE34" s="4"/>
-      <c r="BF34" s="67"/>
-      <c r="BJ34" s="38"/>
-      <c r="BK34" s="4"/>
-      <c r="BL34" s="4"/>
-      <c r="BM34" s="4"/>
-      <c r="BN34" s="4"/>
-    </row>
-    <row r="35" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="38"/>
-      <c r="O35" s="4"/>
-      <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
-      <c r="R35" s="4"/>
-      <c r="S35" s="4"/>
-      <c r="T35" s="4"/>
-      <c r="U35" s="4"/>
-      <c r="AU35" s="4"/>
-      <c r="AV35" s="4"/>
-      <c r="AW35" s="4"/>
-      <c r="AX35" s="4"/>
-      <c r="AY35" s="4"/>
-      <c r="AZ35" s="4"/>
-      <c r="BA35" s="4"/>
-      <c r="BB35" s="4"/>
-      <c r="BC35" s="5"/>
-      <c r="BD35" s="4"/>
-      <c r="BE35" s="4"/>
-      <c r="BF35" s="67"/>
-      <c r="BJ35" s="38"/>
-      <c r="BK35" s="4"/>
-      <c r="BL35" s="4"/>
-      <c r="BM35" s="4"/>
-      <c r="BN35" s="4"/>
-    </row>
-    <row r="36" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N36" s="38"/>
-      <c r="O36" s="4"/>
-      <c r="P36" s="4"/>
-      <c r="Q36" s="4"/>
-      <c r="R36" s="4"/>
-      <c r="S36" s="4"/>
-      <c r="T36" s="4"/>
-      <c r="U36" s="4"/>
-      <c r="V36" s="4"/>
-      <c r="W36" s="4"/>
-      <c r="X36" s="4"/>
-      <c r="Y36" s="4"/>
-      <c r="Z36" s="4"/>
-      <c r="AA36" s="4"/>
-      <c r="AB36" s="4"/>
-      <c r="AC36" s="4"/>
-      <c r="AD36" s="4"/>
-      <c r="AE36" s="4"/>
-      <c r="AF36" s="4"/>
-      <c r="AG36" s="4"/>
-      <c r="AH36" s="4"/>
-      <c r="AI36" s="4"/>
-      <c r="AJ36" s="4"/>
-      <c r="AK36" s="4"/>
-      <c r="AL36" s="4"/>
-      <c r="AM36" s="4"/>
-      <c r="AN36" s="4"/>
-      <c r="AO36" s="4"/>
-      <c r="AP36" s="4"/>
-      <c r="AQ36" s="4"/>
-      <c r="AR36" s="4"/>
-      <c r="AS36" s="4"/>
-      <c r="AT36" s="4"/>
-      <c r="AU36" s="4"/>
-      <c r="AV36" s="4"/>
-      <c r="AW36" s="4"/>
-      <c r="AX36" s="4"/>
-      <c r="AY36" s="4"/>
-      <c r="AZ36" s="4"/>
-      <c r="BA36" s="4"/>
-      <c r="BB36" s="4"/>
-      <c r="BC36" s="5"/>
-      <c r="BD36" s="4"/>
-      <c r="BE36" s="4"/>
-      <c r="BF36" s="67"/>
-      <c r="BJ36" s="38"/>
-      <c r="BK36" s="4"/>
-    </row>
-    <row r="37" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N37" s="38"/>
-      <c r="O37" s="4"/>
-      <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
-      <c r="R37" s="4"/>
-      <c r="S37" s="4"/>
-      <c r="T37" s="4"/>
-      <c r="U37" s="4"/>
-      <c r="V37" s="4"/>
-      <c r="W37" s="4"/>
-      <c r="X37" s="4"/>
-      <c r="Y37" s="4"/>
-      <c r="Z37" s="4"/>
-      <c r="AA37" s="4"/>
-      <c r="AB37" s="4"/>
-      <c r="AC37" s="4"/>
-      <c r="AD37" s="4"/>
-      <c r="AE37" s="4"/>
-      <c r="AF37" s="4"/>
-      <c r="AG37" s="4"/>
-      <c r="AH37" s="4"/>
-      <c r="AI37" s="4"/>
-      <c r="AJ37" s="4"/>
-      <c r="AK37" s="4"/>
-      <c r="AL37" s="4"/>
-      <c r="AM37" s="4"/>
-      <c r="AN37" s="4"/>
-      <c r="AO37" s="4"/>
-      <c r="AP37" s="4"/>
-      <c r="AQ37" s="4"/>
-      <c r="AR37" s="4"/>
-      <c r="AS37" s="4"/>
-      <c r="AT37" s="4"/>
-      <c r="AU37" s="4"/>
-      <c r="AV37" s="4"/>
-      <c r="AW37" s="4"/>
-      <c r="AX37" s="4"/>
-      <c r="AY37" s="4"/>
-      <c r="AZ37" s="4"/>
-      <c r="BA37" s="4"/>
-      <c r="BB37" s="4"/>
-      <c r="BC37" s="5"/>
-      <c r="BD37" s="4"/>
-      <c r="BE37" s="4"/>
-      <c r="BF37" s="67"/>
-      <c r="BJ37" s="38"/>
-      <c r="BK37" s="4"/>
-    </row>
-    <row r="38" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N38" s="38"/>
-      <c r="O38" s="4"/>
-      <c r="P38" s="4"/>
-      <c r="Q38" s="4"/>
-      <c r="R38" s="4"/>
-      <c r="S38" s="4"/>
-      <c r="T38" s="4"/>
-      <c r="U38" s="4"/>
-      <c r="V38" s="4"/>
-      <c r="W38" s="4"/>
-      <c r="X38" s="4"/>
-      <c r="Y38" s="4"/>
-      <c r="Z38" s="4"/>
-      <c r="AA38" s="4"/>
-      <c r="AB38" s="4"/>
-      <c r="AC38" s="4"/>
-      <c r="AD38" s="4"/>
-      <c r="AE38" s="4"/>
-      <c r="AF38" s="4"/>
-      <c r="AG38" s="4"/>
-      <c r="AH38" s="4"/>
-      <c r="AI38" s="4"/>
-      <c r="AJ38" s="4"/>
-      <c r="AK38" s="4"/>
-      <c r="AL38" s="4"/>
-      <c r="AM38" s="4"/>
-      <c r="AN38" s="4"/>
-      <c r="AO38" s="4"/>
-      <c r="AP38" s="4"/>
-      <c r="AQ38" s="4"/>
-      <c r="AR38" s="4"/>
-      <c r="AS38" s="4"/>
-      <c r="AT38" s="4"/>
-      <c r="AU38" s="4"/>
-      <c r="AV38" s="4"/>
-      <c r="AW38" s="4"/>
-      <c r="AX38" s="4"/>
-      <c r="AY38" s="4"/>
-      <c r="AZ38" s="4"/>
-      <c r="BA38" s="4"/>
-      <c r="BB38" s="4"/>
-      <c r="BC38" s="5"/>
-      <c r="BD38" s="4"/>
-      <c r="BE38" s="4"/>
-      <c r="BF38" s="67"/>
-      <c r="BJ38" s="38"/>
-      <c r="BK38" s="4"/>
-    </row>
-    <row r="39" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N39" s="38"/>
-      <c r="O39" s="4"/>
-      <c r="P39" s="4"/>
-      <c r="Q39" s="4"/>
-      <c r="R39" s="4"/>
-      <c r="S39" s="4"/>
-      <c r="T39" s="4"/>
-      <c r="U39" s="4"/>
-      <c r="V39" s="4"/>
-      <c r="W39" s="4"/>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="4"/>
-      <c r="Z39" s="4"/>
-      <c r="AA39" s="4"/>
-      <c r="AB39" s="4"/>
-      <c r="AC39" s="4"/>
-      <c r="AD39" s="4"/>
-      <c r="AE39" s="4"/>
-      <c r="AF39" s="4"/>
-      <c r="AG39" s="4"/>
-      <c r="AH39" s="4"/>
-      <c r="AI39" s="4"/>
-      <c r="AJ39" s="4"/>
-      <c r="AK39" s="4"/>
-      <c r="AL39" s="4"/>
-      <c r="AM39" s="4"/>
-      <c r="AN39" s="4"/>
-      <c r="AO39" s="4"/>
-      <c r="AP39" s="4"/>
-      <c r="AQ39" s="4"/>
-      <c r="AR39" s="4"/>
-      <c r="AS39" s="4"/>
-      <c r="AT39" s="4"/>
-      <c r="AU39" s="4"/>
-      <c r="AV39" s="4"/>
-      <c r="AW39" s="4"/>
-      <c r="AX39" s="4"/>
-      <c r="AY39" s="4"/>
-      <c r="AZ39" s="4"/>
-      <c r="BA39" s="4"/>
-      <c r="BB39" s="4"/>
-      <c r="BC39" s="5"/>
-      <c r="BD39" s="4"/>
-      <c r="BE39" s="4"/>
-      <c r="BF39" s="67"/>
-      <c r="BJ39" s="38"/>
-      <c r="BK39" s="4"/>
-    </row>
-    <row r="40" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N40" s="38"/>
-      <c r="O40" s="4"/>
-      <c r="P40" s="4"/>
-      <c r="Q40" s="4"/>
-      <c r="R40" s="4"/>
-      <c r="S40" s="4"/>
-      <c r="T40" s="4"/>
-      <c r="U40" s="4"/>
-      <c r="V40" s="4"/>
-      <c r="W40" s="4"/>
-      <c r="X40" s="4"/>
-      <c r="Y40" s="4"/>
-      <c r="Z40" s="4"/>
-      <c r="AA40" s="4"/>
-      <c r="AB40" s="4"/>
-      <c r="AC40" s="4"/>
-      <c r="AD40" s="4"/>
-      <c r="AE40" s="4"/>
-      <c r="AF40" s="4"/>
-      <c r="AG40" s="4"/>
-      <c r="AH40" s="4"/>
-      <c r="AI40" s="4"/>
-      <c r="AJ40" s="4"/>
-      <c r="AK40" s="4"/>
-      <c r="AL40" s="4"/>
-      <c r="AM40" s="4"/>
-      <c r="AN40" s="4"/>
-      <c r="AO40" s="4"/>
-      <c r="AP40" s="4"/>
-      <c r="AQ40" s="4"/>
-      <c r="AR40" s="4"/>
-      <c r="AS40" s="4"/>
-      <c r="AT40" s="4"/>
-      <c r="AU40" s="4"/>
-      <c r="AV40" s="4"/>
-      <c r="AW40" s="4"/>
-      <c r="AX40" s="4"/>
-      <c r="AY40" s="4"/>
-      <c r="AZ40" s="4"/>
-      <c r="BA40" s="4"/>
-      <c r="BB40" s="4"/>
-      <c r="BC40" s="5"/>
-      <c r="BD40" s="4"/>
-      <c r="BE40" s="4"/>
-      <c r="BF40" s="67"/>
-      <c r="BJ40" s="38"/>
-      <c r="BK40" s="4"/>
-    </row>
-    <row r="41" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N41" s="38"/>
-      <c r="O41" s="4"/>
-      <c r="P41" s="4"/>
-      <c r="Q41" s="4"/>
-      <c r="R41" s="4"/>
-      <c r="S41" s="4"/>
-      <c r="T41" s="4"/>
-      <c r="U41" s="4"/>
-      <c r="V41" s="4"/>
-      <c r="W41" s="4"/>
-      <c r="X41" s="4"/>
-      <c r="Y41" s="4"/>
-      <c r="Z41" s="4"/>
-      <c r="AA41" s="4"/>
-      <c r="AB41" s="4"/>
-      <c r="AC41" s="4"/>
-      <c r="AD41" s="4"/>
-      <c r="AE41" s="4"/>
-      <c r="AF41" s="4"/>
-      <c r="AG41" s="4"/>
-      <c r="AH41" s="4"/>
-      <c r="AI41" s="4"/>
-      <c r="AJ41" s="4"/>
-      <c r="AK41" s="4"/>
-      <c r="AL41" s="4"/>
-      <c r="AM41" s="4"/>
-      <c r="AN41" s="4"/>
-      <c r="AO41" s="4"/>
-      <c r="AP41" s="4"/>
-      <c r="AQ41" s="4"/>
-      <c r="AR41" s="4"/>
-      <c r="AS41" s="4"/>
-      <c r="AT41" s="4"/>
-      <c r="AU41" s="4"/>
-      <c r="AV41" s="4"/>
-      <c r="AW41" s="4"/>
-      <c r="AX41" s="48"/>
-      <c r="AY41" s="4"/>
-      <c r="AZ41" s="4"/>
-      <c r="BA41" s="4"/>
-      <c r="BB41" s="4"/>
-      <c r="BC41" s="5"/>
-      <c r="BD41" s="4"/>
-      <c r="BE41" s="4"/>
-      <c r="BF41" s="67"/>
-      <c r="BJ41" s="38"/>
-      <c r="BK41" s="4"/>
-    </row>
-    <row r="42" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N42" s="38"/>
-      <c r="O42" s="4"/>
-      <c r="P42" s="4"/>
-      <c r="Q42" s="4"/>
-      <c r="R42" s="4"/>
-      <c r="S42" s="4"/>
-      <c r="T42" s="4"/>
-      <c r="U42" s="4"/>
-      <c r="V42" s="4"/>
-      <c r="W42" s="4"/>
-      <c r="X42" s="4"/>
-      <c r="Y42" s="4"/>
-      <c r="Z42" s="4"/>
-      <c r="AA42" s="4"/>
-      <c r="AB42" s="4"/>
-      <c r="AC42" s="4"/>
-      <c r="AD42" s="4"/>
-      <c r="AE42" s="4"/>
-      <c r="AF42" s="4"/>
-      <c r="AG42" s="4"/>
-      <c r="AH42" s="4"/>
-      <c r="AI42" s="4"/>
-      <c r="AJ42" s="4"/>
-      <c r="AK42" s="4"/>
-      <c r="AL42" s="4"/>
-      <c r="AM42" s="4"/>
-      <c r="AN42" s="4"/>
-      <c r="AO42" s="4"/>
-      <c r="AP42" s="4"/>
-      <c r="AQ42" s="4"/>
-      <c r="AR42" s="4"/>
-      <c r="AS42" s="4"/>
-      <c r="AT42" s="4"/>
-      <c r="AU42" s="4"/>
-      <c r="AV42" s="4"/>
-      <c r="AW42" s="4"/>
-      <c r="AX42" s="48"/>
-      <c r="AY42" s="4"/>
-      <c r="AZ42" s="4"/>
-      <c r="BA42" s="4"/>
-      <c r="BB42" s="4"/>
-      <c r="BC42" s="5"/>
-      <c r="BD42" s="4"/>
-      <c r="BE42" s="4"/>
-      <c r="BF42" s="67"/>
-      <c r="BJ42" s="38"/>
-      <c r="BK42" s="4"/>
-    </row>
-    <row r="43" spans="1:66" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N43" s="38"/>
-      <c r="O43" s="4"/>
-      <c r="P43" s="4"/>
-      <c r="Q43" s="4"/>
-      <c r="R43" s="4"/>
-      <c r="S43" s="4"/>
-      <c r="T43" s="4"/>
-      <c r="U43" s="4"/>
-      <c r="V43" s="6"/>
-      <c r="W43" s="45"/>
-      <c r="X43" s="45"/>
-      <c r="Y43" s="45"/>
-      <c r="Z43" s="6"/>
-      <c r="AA43" s="6"/>
-      <c r="AB43" s="6"/>
-      <c r="AC43" s="6"/>
-      <c r="AD43" s="6"/>
-      <c r="AE43" s="6"/>
-      <c r="AF43" s="6"/>
-      <c r="AG43" s="6"/>
-      <c r="AH43" s="6"/>
-      <c r="AI43" s="6"/>
-      <c r="AJ43" s="6"/>
-      <c r="AK43" s="6"/>
-      <c r="AL43" s="6"/>
-      <c r="AM43" s="6"/>
-      <c r="AN43" s="6"/>
-      <c r="AO43" s="6"/>
-      <c r="AP43" s="6"/>
-      <c r="AQ43" s="6"/>
-      <c r="AR43" s="6"/>
-      <c r="AS43" s="6"/>
-      <c r="AT43" s="6"/>
-      <c r="AU43" s="6"/>
-      <c r="AV43" s="45"/>
-      <c r="AW43" s="45"/>
-      <c r="AX43" s="49"/>
-      <c r="AY43" s="6"/>
-      <c r="AZ43" s="6"/>
-      <c r="BA43" s="6"/>
-      <c r="BB43" s="6"/>
-      <c r="BC43" s="7"/>
-      <c r="BD43" s="4"/>
-      <c r="BE43" s="4"/>
-      <c r="BF43" s="67"/>
-      <c r="BJ43" s="38"/>
-      <c r="BK43" s="4"/>
-    </row>
-    <row r="44" spans="1:66" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N44" s="38"/>
-      <c r="O44" s="4"/>
-      <c r="P44" s="4"/>
-      <c r="Q44" s="4"/>
-      <c r="R44" s="4"/>
-      <c r="S44" s="4"/>
-      <c r="T44" s="4"/>
-      <c r="U44" s="5"/>
-      <c r="V44" s="22"/>
-      <c r="W44" s="46"/>
-      <c r="X44" s="73"/>
-      <c r="Y44" s="46"/>
-      <c r="Z44" s="19"/>
-      <c r="AA44" s="19"/>
-      <c r="AB44" s="19"/>
-      <c r="AC44" s="19"/>
-      <c r="AD44" s="19"/>
-      <c r="AE44" s="19"/>
-      <c r="AF44" s="19"/>
-      <c r="AG44" s="19"/>
-      <c r="AH44" s="19"/>
-      <c r="AI44" s="19"/>
-      <c r="AJ44" s="19"/>
-      <c r="AK44" s="19"/>
-      <c r="AL44" s="19"/>
-      <c r="AM44" s="19"/>
-      <c r="AN44" s="19"/>
-      <c r="AO44" s="19"/>
-      <c r="AP44" s="19"/>
-      <c r="AQ44" s="19"/>
-      <c r="AR44" s="19"/>
-      <c r="AS44" s="41"/>
-      <c r="AT44" s="43"/>
-      <c r="AU44" s="19"/>
-      <c r="AV44" s="74"/>
-      <c r="AW44" s="46"/>
-      <c r="AX44" s="47"/>
-      <c r="AY44" s="19"/>
-      <c r="AZ44" s="19"/>
-      <c r="BA44" s="19"/>
-      <c r="BB44" s="19"/>
-      <c r="BC44" s="20"/>
-      <c r="BD44" s="4"/>
-      <c r="BE44" s="4"/>
-      <c r="BF44" s="67"/>
-      <c r="BJ44" s="38"/>
-      <c r="BK44" s="4"/>
-    </row>
-    <row r="45" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N45" s="38"/>
-      <c r="O45" s="4"/>
-      <c r="P45" s="4"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
-      <c r="T45" s="4"/>
-      <c r="U45" s="5"/>
-      <c r="V45" s="38"/>
-      <c r="W45" s="4"/>
-      <c r="X45" s="58"/>
-      <c r="Y45" s="4"/>
-      <c r="Z45" s="4"/>
-      <c r="AA45" s="4"/>
-      <c r="AB45" s="4"/>
-      <c r="AC45" s="4"/>
-      <c r="AD45" s="4"/>
-      <c r="AE45" s="4"/>
-      <c r="AF45" s="4"/>
-      <c r="AG45" s="4"/>
-      <c r="AH45" s="4"/>
-      <c r="AI45" s="4"/>
-      <c r="AJ45" s="4"/>
-      <c r="AK45" s="4"/>
-      <c r="AL45" s="4"/>
-      <c r="AM45" s="4"/>
-      <c r="AN45" s="4"/>
-      <c r="AO45" s="4"/>
-      <c r="AP45" s="4"/>
-      <c r="AQ45" s="54"/>
-      <c r="AR45" s="55"/>
-      <c r="AS45" s="56"/>
-      <c r="AT45" s="57"/>
-      <c r="AU45" s="55"/>
-      <c r="AV45" s="55"/>
-      <c r="AW45" s="4"/>
-      <c r="AX45" s="39"/>
-      <c r="AY45" s="4"/>
-      <c r="AZ45" s="4"/>
-      <c r="BA45" s="4"/>
-      <c r="BB45" s="4"/>
-      <c r="BC45" s="52"/>
-      <c r="BD45" s="53"/>
-      <c r="BE45" s="4"/>
-      <c r="BF45" s="67"/>
-      <c r="BJ45" s="38"/>
-      <c r="BK45" s="4"/>
-    </row>
-    <row r="46" spans="1:66" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N46" s="38"/>
-      <c r="O46" s="4"/>
-      <c r="P46" s="4"/>
-      <c r="Q46" s="4"/>
-      <c r="R46" s="4"/>
-      <c r="S46" s="4"/>
-      <c r="T46" s="4"/>
-      <c r="U46" s="5"/>
-      <c r="V46" s="38"/>
-      <c r="W46" s="4"/>
-      <c r="X46" s="58"/>
-      <c r="Y46" s="4"/>
-      <c r="Z46" s="4"/>
-      <c r="AA46" s="4"/>
-      <c r="AB46" s="4"/>
-      <c r="AC46" s="4"/>
-      <c r="AD46" s="4"/>
-      <c r="AE46" s="4"/>
-      <c r="AF46" s="4"/>
-      <c r="AG46" s="4"/>
-      <c r="AH46" s="4"/>
-      <c r="AI46" s="4"/>
-      <c r="AJ46" s="4"/>
-      <c r="AK46" s="4"/>
-      <c r="AL46" s="4"/>
-      <c r="AM46" s="4"/>
-      <c r="AN46" s="4"/>
-      <c r="AO46" s="4"/>
-      <c r="AP46" s="4"/>
-      <c r="AQ46" s="58"/>
-      <c r="AR46" s="4"/>
-      <c r="AS46" s="42"/>
-      <c r="AT46" s="44"/>
-      <c r="AU46" s="13"/>
-      <c r="AV46" s="13"/>
-      <c r="AW46" s="13"/>
-      <c r="AX46" s="40"/>
-      <c r="AY46" s="4"/>
-      <c r="AZ46" s="4"/>
-      <c r="BA46" s="4"/>
-      <c r="BB46" s="4"/>
-      <c r="BC46" s="52"/>
-      <c r="BD46" s="53"/>
-      <c r="BE46" s="4"/>
-      <c r="BF46" s="67"/>
-      <c r="BJ46" s="38"/>
-      <c r="BK46" s="4"/>
-    </row>
-    <row r="47" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="N47" s="38"/>
-      <c r="O47" s="4"/>
-      <c r="P47" s="4"/>
-      <c r="Q47" s="4"/>
-      <c r="R47" s="4"/>
-      <c r="S47" s="4"/>
-      <c r="T47" s="4"/>
-      <c r="U47" s="50"/>
-      <c r="V47" s="51"/>
-      <c r="W47" s="4"/>
-      <c r="X47" s="58"/>
-      <c r="Y47" s="4"/>
-      <c r="Z47" s="4"/>
-      <c r="AA47" s="4"/>
-      <c r="AB47" s="4"/>
-      <c r="AC47" s="4"/>
-      <c r="AD47" s="4"/>
-      <c r="AE47" s="4"/>
-      <c r="AF47" s="4"/>
-      <c r="AG47" s="4"/>
-      <c r="AH47" s="4"/>
-      <c r="AI47" s="4"/>
-      <c r="AJ47" s="4"/>
-      <c r="AK47" s="4"/>
-      <c r="AL47" s="4"/>
-      <c r="AM47" s="4"/>
-      <c r="AN47" s="4"/>
-      <c r="AO47" s="4"/>
-      <c r="AP47" s="4"/>
-      <c r="AQ47" s="58"/>
-      <c r="AR47" s="4"/>
-      <c r="AS47" s="4"/>
-      <c r="AT47" s="4"/>
-      <c r="AU47" s="4"/>
-      <c r="AV47" s="4"/>
-      <c r="AW47" s="4"/>
-      <c r="AX47" s="4"/>
-      <c r="AY47" s="4"/>
-      <c r="AZ47" s="4"/>
-      <c r="BA47" s="4"/>
-      <c r="BB47" s="4"/>
-      <c r="BC47" s="52"/>
-      <c r="BD47" s="53"/>
-      <c r="BE47" s="4"/>
-      <c r="BF47" s="67"/>
-      <c r="BJ47" s="38"/>
-      <c r="BK47" s="4"/>
-    </row>
-    <row r="48" spans="1:66" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N48" s="38"/>
-      <c r="O48" s="4"/>
-      <c r="P48" s="4"/>
-      <c r="Q48" s="4"/>
-      <c r="R48" s="4"/>
-      <c r="S48" s="4"/>
-      <c r="T48" s="4"/>
-      <c r="U48" s="50"/>
-      <c r="V48" s="51"/>
-      <c r="W48" s="4"/>
-      <c r="X48" s="59"/>
-      <c r="Y48" s="60"/>
-      <c r="Z48" s="60"/>
-      <c r="AA48" s="60"/>
-      <c r="AB48" s="60"/>
-      <c r="AC48" s="60"/>
-      <c r="AD48" s="60"/>
-      <c r="AE48" s="60"/>
-      <c r="AF48" s="60"/>
-      <c r="AG48" s="60"/>
-      <c r="AH48" s="60"/>
-      <c r="AI48" s="60"/>
-      <c r="AJ48" s="60"/>
-      <c r="AK48" s="60"/>
-      <c r="AL48" s="60"/>
-      <c r="AM48" s="60"/>
-      <c r="AN48" s="60"/>
-      <c r="AO48" s="60"/>
-      <c r="AP48" s="60"/>
-      <c r="AQ48" s="59"/>
-      <c r="AR48" s="60"/>
-      <c r="AS48" s="60"/>
-      <c r="AT48" s="60"/>
-      <c r="AU48" s="60"/>
-      <c r="AV48" s="60"/>
-      <c r="AW48" s="60"/>
-      <c r="AX48" s="60"/>
-      <c r="AY48" s="60"/>
-      <c r="AZ48" s="60"/>
-      <c r="BA48" s="60"/>
-      <c r="BB48" s="60"/>
-      <c r="BC48" s="69"/>
-      <c r="BD48" s="70"/>
-      <c r="BE48" s="60"/>
-      <c r="BF48" s="71"/>
-      <c r="BJ48" s="38"/>
-      <c r="BK48" s="4"/>
-    </row>
-    <row r="49" spans="14:63" x14ac:dyDescent="0.25">
-      <c r="N49" s="38"/>
-      <c r="O49" s="4"/>
-      <c r="P49" s="4"/>
-      <c r="Q49" s="4"/>
-      <c r="R49" s="4"/>
-      <c r="S49" s="4"/>
-      <c r="T49" s="4"/>
-      <c r="U49" s="50"/>
-      <c r="V49" s="51"/>
-      <c r="W49" s="4"/>
-      <c r="X49" s="4"/>
-      <c r="Y49" s="4"/>
-      <c r="Z49" s="4"/>
-      <c r="AA49" s="4"/>
-      <c r="AB49" s="4"/>
-      <c r="AC49" s="4"/>
-      <c r="AD49" s="4"/>
-      <c r="AE49" s="4"/>
-      <c r="AF49" s="4"/>
-      <c r="AG49" s="4"/>
-      <c r="AH49" s="4"/>
-      <c r="AI49" s="4"/>
-      <c r="AJ49" s="4"/>
-      <c r="AK49" s="4"/>
-      <c r="AL49" s="4"/>
-      <c r="AM49" s="4"/>
-      <c r="AN49" s="4"/>
-      <c r="AO49" s="4"/>
-      <c r="AP49" s="4"/>
-      <c r="AQ49" s="4"/>
-      <c r="AR49" s="4"/>
-      <c r="AS49" s="4"/>
-      <c r="AT49" s="4"/>
-      <c r="AU49" s="4"/>
-      <c r="AV49" s="4"/>
-      <c r="AW49" s="4"/>
-      <c r="AX49" s="4"/>
-      <c r="AY49" s="4"/>
-      <c r="AZ49" s="4"/>
-      <c r="BA49" s="4"/>
-      <c r="BB49" s="4"/>
-      <c r="BC49" s="52"/>
-      <c r="BD49" s="53"/>
-      <c r="BJ49" s="38"/>
-      <c r="BK49" s="4"/>
-    </row>
-    <row r="50" spans="14:63" x14ac:dyDescent="0.25">
-      <c r="N50" s="38"/>
-      <c r="O50" s="4"/>
-      <c r="P50" s="4"/>
-      <c r="Q50" s="4"/>
-      <c r="R50" s="4"/>
-      <c r="S50" s="4"/>
-      <c r="T50" s="4"/>
-      <c r="U50" s="5"/>
-      <c r="V50" s="38"/>
-      <c r="W50" s="4"/>
-      <c r="X50" s="4"/>
-      <c r="Y50" s="4"/>
-      <c r="Z50" s="4"/>
-      <c r="AA50" s="4"/>
-      <c r="AB50" s="4"/>
-      <c r="AC50" s="4"/>
-      <c r="AD50" s="4"/>
-      <c r="AE50" s="4"/>
-      <c r="AF50" s="4"/>
-      <c r="AG50" s="4"/>
-      <c r="AH50" s="4"/>
-      <c r="AI50" s="4"/>
-      <c r="AJ50" s="4"/>
-      <c r="AK50" s="4"/>
-      <c r="AL50" s="4"/>
-      <c r="AM50" s="4"/>
-      <c r="AN50" s="4"/>
-      <c r="AO50" s="4"/>
-      <c r="AP50" s="4"/>
-      <c r="AQ50" s="4"/>
-      <c r="AR50" s="4"/>
-      <c r="AS50" s="4"/>
-      <c r="AT50" s="4"/>
-      <c r="AU50" s="4"/>
-      <c r="AV50" s="4"/>
-      <c r="AW50" s="4"/>
-      <c r="AX50" s="4"/>
-      <c r="AY50" s="4"/>
-      <c r="AZ50" s="4"/>
-      <c r="BA50" s="4"/>
-      <c r="BB50" s="4"/>
-      <c r="BC50" s="52"/>
-      <c r="BD50" s="53"/>
-      <c r="BJ50" s="38"/>
-      <c r="BK50" s="4"/>
-    </row>
-    <row r="51" spans="14:63" x14ac:dyDescent="0.25">
-      <c r="N51" s="38"/>
-      <c r="O51" s="4"/>
-      <c r="P51" s="4"/>
-      <c r="Q51" s="4"/>
-      <c r="R51" s="4"/>
-      <c r="S51" s="4"/>
-      <c r="T51" s="4"/>
-      <c r="U51" s="5"/>
-      <c r="V51" s="38"/>
-      <c r="W51" s="4"/>
-      <c r="X51" s="4"/>
-      <c r="Y51" s="4"/>
-      <c r="Z51" s="4"/>
-      <c r="AA51" s="4"/>
-      <c r="AB51" s="4"/>
-      <c r="AC51" s="4"/>
-      <c r="AD51" s="4"/>
-      <c r="AE51" s="4"/>
-      <c r="AF51" s="4"/>
-      <c r="AG51" s="4"/>
-      <c r="AH51" s="4"/>
-      <c r="AI51" s="4"/>
-      <c r="AJ51" s="4"/>
-      <c r="AK51" s="4"/>
-      <c r="AL51" s="4"/>
-      <c r="AM51" s="4"/>
-      <c r="AN51" s="4"/>
-      <c r="AO51" s="4"/>
-      <c r="AP51" s="4"/>
-      <c r="AQ51" s="4"/>
-      <c r="AR51" s="4"/>
-      <c r="AS51" s="4"/>
-      <c r="AT51" s="4"/>
-      <c r="AU51" s="4"/>
-      <c r="AV51" s="4"/>
-      <c r="AW51" s="4"/>
-      <c r="AX51" s="4"/>
-      <c r="AY51" s="4"/>
-      <c r="AZ51" s="4"/>
-      <c r="BA51" s="4"/>
-      <c r="BB51" s="4"/>
-      <c r="BC51" s="52"/>
-      <c r="BD51" s="53"/>
-      <c r="BJ51" s="38"/>
-      <c r="BK51" s="4"/>
-    </row>
-    <row r="52" spans="14:63" x14ac:dyDescent="0.25">
-      <c r="N52" s="38"/>
-      <c r="O52" s="4"/>
-      <c r="P52" s="4"/>
-      <c r="Q52" s="4"/>
-      <c r="R52" s="4"/>
-      <c r="S52" s="4"/>
-      <c r="T52" s="4"/>
-      <c r="U52" s="5"/>
-      <c r="V52" s="38"/>
-      <c r="W52" s="4"/>
-      <c r="X52" s="4"/>
-      <c r="Y52" s="4"/>
-      <c r="Z52" s="4"/>
-      <c r="AA52" s="4"/>
-      <c r="AB52" s="4"/>
-      <c r="AC52" s="4"/>
-      <c r="AD52" s="4"/>
-      <c r="AE52" s="4"/>
-      <c r="AF52" s="4"/>
-      <c r="AG52" s="4"/>
-      <c r="AH52" s="4"/>
-      <c r="AI52" s="4"/>
-      <c r="AJ52" s="4"/>
-      <c r="AK52" s="4"/>
-      <c r="AL52" s="4"/>
-      <c r="AM52" s="4"/>
-      <c r="AN52" s="4"/>
-      <c r="AO52" s="4"/>
-      <c r="AP52" s="4"/>
-      <c r="AQ52" s="4"/>
-      <c r="AR52" s="4"/>
-      <c r="AS52" s="4"/>
-      <c r="AT52" s="4"/>
-      <c r="AU52" s="4"/>
-      <c r="AV52" s="4"/>
-      <c r="AW52" s="4"/>
-      <c r="AX52" s="4"/>
-      <c r="AY52" s="4"/>
-      <c r="AZ52" s="4"/>
-      <c r="BA52" s="4"/>
-      <c r="BB52" s="4"/>
-      <c r="BC52" s="52"/>
-      <c r="BD52" s="53"/>
-      <c r="BJ52" s="38"/>
-      <c r="BK52" s="4"/>
-    </row>
-    <row r="53" spans="14:63" x14ac:dyDescent="0.25">
-      <c r="N53" s="38"/>
-      <c r="O53" s="4"/>
-      <c r="P53" s="4"/>
-      <c r="Q53" s="4"/>
-      <c r="R53" s="4"/>
-      <c r="S53" s="4"/>
-      <c r="T53" s="4"/>
-      <c r="U53" s="5"/>
-      <c r="V53" s="38"/>
-      <c r="W53" s="4"/>
-      <c r="X53" s="4"/>
-      <c r="Y53" s="4"/>
-      <c r="Z53" s="4"/>
-      <c r="AA53" s="4"/>
-      <c r="AB53" s="4"/>
-      <c r="AC53" s="4"/>
-      <c r="AD53" s="4"/>
-      <c r="AE53" s="4"/>
-      <c r="AF53" s="4"/>
-      <c r="AG53" s="4"/>
-      <c r="AH53" s="4"/>
-      <c r="AI53" s="4"/>
-      <c r="AJ53" s="4"/>
-      <c r="AK53" s="4"/>
-      <c r="AL53" s="4"/>
-      <c r="AM53" s="4"/>
-      <c r="AN53" s="4"/>
-      <c r="AO53" s="4"/>
-      <c r="AP53" s="4"/>
-      <c r="AQ53" s="4"/>
-      <c r="AR53" s="4"/>
-      <c r="AS53" s="4"/>
-      <c r="AT53" s="4"/>
-      <c r="AU53" s="4"/>
-      <c r="AV53" s="4"/>
-      <c r="AW53" s="4"/>
-      <c r="AX53" s="4"/>
-      <c r="AY53" s="4"/>
-      <c r="AZ53" s="4"/>
-      <c r="BA53" s="4"/>
-      <c r="BB53" s="4"/>
-      <c r="BC53" s="75"/>
-      <c r="BJ53" s="38"/>
-      <c r="BK53" s="4"/>
-    </row>
-    <row r="54" spans="14:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N54" s="21"/>
-      <c r="O54" s="6"/>
-      <c r="P54" s="6"/>
-      <c r="Q54" s="6"/>
-      <c r="R54" s="6"/>
-      <c r="S54" s="6"/>
-      <c r="T54" s="6"/>
-      <c r="U54" s="7"/>
-      <c r="V54" s="76"/>
-      <c r="W54" s="77"/>
-      <c r="X54" s="77"/>
-      <c r="Y54" s="77"/>
-      <c r="Z54" s="77"/>
-      <c r="AA54" s="77"/>
-      <c r="AB54" s="77"/>
-      <c r="AC54" s="77"/>
-      <c r="AD54" s="77"/>
-      <c r="AE54" s="77"/>
-      <c r="AF54" s="77"/>
-      <c r="AG54" s="77"/>
-      <c r="AH54" s="77"/>
-      <c r="AI54" s="77"/>
-      <c r="AJ54" s="77"/>
-      <c r="AK54" s="77"/>
-      <c r="AL54" s="77"/>
-      <c r="AM54" s="77"/>
-      <c r="AN54" s="77"/>
-      <c r="AO54" s="77"/>
-      <c r="AP54" s="77"/>
-      <c r="AQ54" s="77"/>
-      <c r="AR54" s="77"/>
-      <c r="AS54" s="77"/>
-      <c r="AT54" s="77"/>
-      <c r="AU54" s="77"/>
-      <c r="AV54" s="77"/>
-      <c r="AW54" s="77"/>
-      <c r="AX54" s="77"/>
-      <c r="AY54" s="77"/>
-      <c r="AZ54" s="77"/>
-      <c r="BA54" s="77"/>
-      <c r="BB54" s="77"/>
-      <c r="BC54" s="78"/>
-      <c r="BJ54" s="38"/>
-      <c r="BK54" s="4"/>
-    </row>
-    <row r="55" spans="14:63" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="BC55" s="79"/>
-      <c r="BJ55" s="38"/>
-      <c r="BK55" s="4"/>
+      <c r="BC32" s="4"/>
+      <c r="BF32" s="65"/>
+      <c r="BJ32" s="37"/>
+    </row>
+    <row r="33" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="M33" s="4"/>
+      <c r="BC33" s="4"/>
+      <c r="BF33" s="65"/>
+      <c r="BJ33" s="37"/>
+    </row>
+    <row r="34" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="M34" s="4"/>
+      <c r="BC34" s="4"/>
+      <c r="BF34" s="65"/>
+      <c r="BJ34" s="37"/>
+    </row>
+    <row r="35" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N35" s="37"/>
+      <c r="BC35" s="4"/>
+      <c r="BF35" s="65"/>
+      <c r="BJ35" s="37"/>
+    </row>
+    <row r="36" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N36" s="37"/>
+      <c r="BC36" s="4"/>
+      <c r="BF36" s="65"/>
+      <c r="BJ36" s="37"/>
+    </row>
+    <row r="37" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N37" s="37"/>
+      <c r="BC37" s="4"/>
+      <c r="BF37" s="65"/>
+      <c r="BJ37" s="37"/>
+    </row>
+    <row r="38" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N38" s="37"/>
+      <c r="BC38" s="4"/>
+      <c r="BF38" s="65"/>
+      <c r="BJ38" s="37"/>
+    </row>
+    <row r="39" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N39" s="37"/>
+      <c r="BC39" s="4"/>
+      <c r="BF39" s="65"/>
+      <c r="BJ39" s="37"/>
+    </row>
+    <row r="40" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N40" s="37"/>
+      <c r="BC40" s="4"/>
+      <c r="BF40" s="65"/>
+      <c r="BJ40" s="37"/>
+    </row>
+    <row r="41" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N41" s="37"/>
+      <c r="AX41" s="47"/>
+      <c r="BC41" s="4"/>
+      <c r="BF41" s="65"/>
+      <c r="BJ41" s="37"/>
+    </row>
+    <row r="42" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N42" s="37"/>
+      <c r="AX42" s="47"/>
+      <c r="BC42" s="4"/>
+      <c r="BF42" s="65"/>
+      <c r="BJ42" s="37"/>
+    </row>
+    <row r="43" spans="13:62" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N43" s="37"/>
+      <c r="V43" s="5"/>
+      <c r="W43" s="44"/>
+      <c r="X43" s="44"/>
+      <c r="Y43" s="44"/>
+      <c r="Z43" s="5"/>
+      <c r="AA43" s="5"/>
+      <c r="AB43" s="5"/>
+      <c r="AC43" s="5"/>
+      <c r="AD43" s="5"/>
+      <c r="AE43" s="5"/>
+      <c r="AF43" s="5"/>
+      <c r="AG43" s="5"/>
+      <c r="AH43" s="5"/>
+      <c r="AI43" s="5"/>
+      <c r="AJ43" s="5"/>
+      <c r="AK43" s="5"/>
+      <c r="AL43" s="5"/>
+      <c r="AM43" s="5"/>
+      <c r="AN43" s="5"/>
+      <c r="AO43" s="5"/>
+      <c r="AP43" s="5"/>
+      <c r="AQ43" s="5"/>
+      <c r="AR43" s="5"/>
+      <c r="AS43" s="5"/>
+      <c r="AT43" s="5"/>
+      <c r="AU43" s="5"/>
+      <c r="AV43" s="44"/>
+      <c r="AW43" s="44"/>
+      <c r="AX43" s="48"/>
+      <c r="AY43" s="5"/>
+      <c r="AZ43" s="5"/>
+      <c r="BA43" s="5"/>
+      <c r="BB43" s="5"/>
+      <c r="BC43" s="6"/>
+      <c r="BF43" s="65"/>
+      <c r="BJ43" s="37"/>
+    </row>
+    <row r="44" spans="13:62" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N44" s="37"/>
+      <c r="U44" s="4"/>
+      <c r="V44" s="21"/>
+      <c r="W44" s="45"/>
+      <c r="X44" s="70"/>
+      <c r="Y44" s="45"/>
+      <c r="Z44" s="18"/>
+      <c r="AA44" s="18"/>
+      <c r="AB44" s="18"/>
+      <c r="AC44" s="18"/>
+      <c r="AD44" s="18"/>
+      <c r="AE44" s="18"/>
+      <c r="AF44" s="18"/>
+      <c r="AG44" s="18"/>
+      <c r="AH44" s="18"/>
+      <c r="AI44" s="18"/>
+      <c r="AJ44" s="18"/>
+      <c r="AK44" s="18"/>
+      <c r="AL44" s="18"/>
+      <c r="AM44" s="18"/>
+      <c r="AN44" s="18"/>
+      <c r="AO44" s="18"/>
+      <c r="AP44" s="18"/>
+      <c r="AQ44" s="18"/>
+      <c r="AR44" s="18"/>
+      <c r="AS44" s="40"/>
+      <c r="AT44" s="42"/>
+      <c r="AU44" s="18"/>
+      <c r="AV44" s="71"/>
+      <c r="AW44" s="45"/>
+      <c r="AX44" s="46"/>
+      <c r="AY44" s="18"/>
+      <c r="AZ44" s="18"/>
+      <c r="BA44" s="18"/>
+      <c r="BB44" s="18"/>
+      <c r="BC44" s="19"/>
+      <c r="BF44" s="65"/>
+      <c r="BJ44" s="37"/>
+    </row>
+    <row r="45" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N45" s="37"/>
+      <c r="U45" s="4"/>
+      <c r="V45" s="37"/>
+      <c r="X45" s="57"/>
+      <c r="AQ45" s="53"/>
+      <c r="AR45" s="54"/>
+      <c r="AS45" s="55"/>
+      <c r="AT45" s="56"/>
+      <c r="AU45" s="54"/>
+      <c r="AV45" s="54"/>
+      <c r="AX45" s="38"/>
+      <c r="BC45" s="51"/>
+      <c r="BD45" s="52"/>
+      <c r="BF45" s="65"/>
+      <c r="BJ45" s="37"/>
+    </row>
+    <row r="46" spans="13:62" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N46" s="37"/>
+      <c r="U46" s="4"/>
+      <c r="V46" s="37"/>
+      <c r="X46" s="57"/>
+      <c r="AQ46" s="57"/>
+      <c r="AS46" s="41"/>
+      <c r="AT46" s="43"/>
+      <c r="AU46" s="12"/>
+      <c r="AV46" s="12"/>
+      <c r="AW46" s="12"/>
+      <c r="AX46" s="39"/>
+      <c r="BC46" s="51"/>
+      <c r="BD46" s="52"/>
+      <c r="BF46" s="65"/>
+      <c r="BJ46" s="37"/>
+    </row>
+    <row r="47" spans="13:62" x14ac:dyDescent="0.25">
+      <c r="N47" s="37"/>
+      <c r="U47" s="49"/>
+      <c r="V47" s="50"/>
+      <c r="X47" s="57"/>
+      <c r="AQ47" s="57"/>
+      <c r="BC47" s="51"/>
+      <c r="BD47" s="52"/>
+      <c r="BF47" s="65"/>
+      <c r="BJ47" s="37"/>
+    </row>
+    <row r="48" spans="13:62" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N48" s="37"/>
+      <c r="U48" s="49"/>
+      <c r="V48" s="50"/>
+      <c r="X48" s="58"/>
+      <c r="Y48" s="59"/>
+      <c r="Z48" s="59"/>
+      <c r="AA48" s="59"/>
+      <c r="AB48" s="59"/>
+      <c r="AC48" s="59"/>
+      <c r="AD48" s="59"/>
+      <c r="AE48" s="59"/>
+      <c r="AF48" s="59"/>
+      <c r="AG48" s="59"/>
+      <c r="AH48" s="59"/>
+      <c r="AI48" s="59"/>
+      <c r="AJ48" s="59"/>
+      <c r="AK48" s="59"/>
+      <c r="AL48" s="59"/>
+      <c r="AM48" s="59"/>
+      <c r="AN48" s="59"/>
+      <c r="AO48" s="59"/>
+      <c r="AP48" s="59"/>
+      <c r="AQ48" s="58"/>
+      <c r="AR48" s="59"/>
+      <c r="AS48" s="59"/>
+      <c r="AT48" s="59"/>
+      <c r="AU48" s="59"/>
+      <c r="AV48" s="59"/>
+      <c r="AW48" s="59"/>
+      <c r="AX48" s="59"/>
+      <c r="AY48" s="59"/>
+      <c r="AZ48" s="59"/>
+      <c r="BA48" s="59"/>
+      <c r="BB48" s="59"/>
+      <c r="BC48" s="66"/>
+      <c r="BD48" s="67"/>
+      <c r="BE48" s="59"/>
+      <c r="BF48" s="68"/>
+      <c r="BJ48" s="37"/>
+    </row>
+    <row r="49" spans="14:62" x14ac:dyDescent="0.25">
+      <c r="N49" s="37"/>
+      <c r="U49" s="49"/>
+      <c r="V49" s="50"/>
+      <c r="BC49" s="51"/>
+      <c r="BD49" s="52"/>
+      <c r="BJ49" s="37"/>
+    </row>
+    <row r="50" spans="14:62" x14ac:dyDescent="0.25">
+      <c r="N50" s="37"/>
+      <c r="U50" s="4"/>
+      <c r="V50" s="37"/>
+      <c r="BC50" s="51"/>
+      <c r="BD50" s="52"/>
+      <c r="BJ50" s="37"/>
+    </row>
+    <row r="51" spans="14:62" x14ac:dyDescent="0.25">
+      <c r="N51" s="37"/>
+      <c r="U51" s="4"/>
+      <c r="V51" s="37"/>
+      <c r="BC51" s="51"/>
+      <c r="BD51" s="52"/>
+      <c r="BJ51" s="37"/>
+    </row>
+    <row r="52" spans="14:62" x14ac:dyDescent="0.25">
+      <c r="N52" s="37"/>
+      <c r="U52" s="4"/>
+      <c r="V52" s="37"/>
+      <c r="BC52" s="51"/>
+      <c r="BD52" s="52"/>
+      <c r="BJ52" s="37"/>
+    </row>
+    <row r="53" spans="14:62" x14ac:dyDescent="0.25">
+      <c r="N53" s="37"/>
+      <c r="U53" s="4"/>
+      <c r="V53" s="37"/>
+      <c r="BC53" s="72"/>
+      <c r="BJ53" s="37"/>
+    </row>
+    <row r="54" spans="14:62" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N54" s="20"/>
+      <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
+      <c r="Q54" s="5"/>
+      <c r="R54" s="5"/>
+      <c r="S54" s="5"/>
+      <c r="T54" s="5"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="73"/>
+      <c r="W54" s="74"/>
+      <c r="X54" s="74"/>
+      <c r="Y54" s="74"/>
+      <c r="Z54" s="74"/>
+      <c r="AA54" s="74"/>
+      <c r="AB54" s="74"/>
+      <c r="AC54" s="74"/>
+      <c r="AD54" s="74"/>
+      <c r="AE54" s="74"/>
+      <c r="AF54" s="74"/>
+      <c r="AG54" s="74"/>
+      <c r="AH54" s="74"/>
+      <c r="AI54" s="74"/>
+      <c r="AJ54" s="74"/>
+      <c r="AK54" s="74"/>
+      <c r="AL54" s="74"/>
+      <c r="AM54" s="74"/>
+      <c r="AN54" s="74"/>
+      <c r="AO54" s="74"/>
+      <c r="AP54" s="74"/>
+      <c r="AQ54" s="74"/>
+      <c r="AR54" s="74"/>
+      <c r="AS54" s="74"/>
+      <c r="AT54" s="74"/>
+      <c r="AU54" s="74"/>
+      <c r="AV54" s="74"/>
+      <c r="AW54" s="74"/>
+      <c r="AX54" s="74"/>
+      <c r="AY54" s="74"/>
+      <c r="AZ54" s="74"/>
+      <c r="BA54" s="74"/>
+      <c r="BB54" s="74"/>
+      <c r="BC54" s="75"/>
+      <c r="BJ54" s="37"/>
+    </row>
+    <row r="55" spans="14:62" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="BC55" s="76"/>
+      <c r="BJ55" s="37"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>